<commit_message>
added traffic light app_3 works
</commit_message>
<xml_diff>
--- a/objekt_data.xlsx
+++ b/objekt_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -428,6 +428,294 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Titel</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Zigeunerinnen mit Sonnenblumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Künstler*in/Autor*in</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Sichtbare oder genannte Personen</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Entstehungsjahr</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1927</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ort der Entstehung / Nutzung</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Gattung / Genre</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Technik</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Leimfarbe, Rupfen</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Dimensionen</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Kurzbeschreibung</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Motive / Topoi</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Narrative / Diskurse</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Darstellung von alternativen Leben fernab der Mehrheitsgesellschaft. Romantisierung des Landlebens. </t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Historischer Kontext</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Otto Mueller war Mitglied der expressionistischen Künstlergruppe Brücke, die sich bewusst gegen akademische Kunstkonventionen stellte. Er suchte nach Ursprünglichkeit, Einfachheit und "Naturverbundenheit" – Werte, die viele Expressionisten romantisch mit nicht-bürgerlichen oder „exotischen“ Gruppen wie z.B. den Roma verbanden.In den 1920er Jahren, in der Weimarer Republik, waren Romnja gesellschaftlich stark marginalisiert. Sie wurden überwacht, ausgegrenzt und kriminalisiert. Die Tendenzen des aufkommenden Nationalsozialismus sind zur Entstehungszeit des Bilds schon deutlich. Mueller hatte persönliche Kontakte zu einer Roma-Gruppe in Schlesien, mit der er wiederholt reiste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Antiziganistische / Stigmatisierende Elemente</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Agency</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Die Figuren sind nicht karikiert oder grotesk. Darstellung von Fürsorge und Wärme. Kind ist Zentrum einer familiären Handlung. </t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Verknüpfung</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Narrativwandel bei Medienwechsel</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Rezeptionsweg</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Sammlung / Archiv</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Provenienz</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Vorbesitzer: Köln, Galerie Aenne AbelsVorbesitzer: Berlin, Mueller, Maschka</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Literatur</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Neue Kunst in der Orangerie (1929): Vierte große Kunstausstellung Kassel. Ausstellungskatalog. Kassel: Kunstverein Kassel.Barr, Alfred H. (1931): German Painting and Sculpture. Ausstellungskatalog. New York: Museum of Modern Art.Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F. u. a. (Hrsg.) (1931): Museum der Gegenwart. Zeitschrift der deutschen Museen für neuere Kunst, 1., 2. Berlin.Allgemeine deutsche Kunstausstellung (1946). [o. Verlagsort].Balzer, Wolfgang (1947): Otto Mueller, 1874–1930. Gemälde, Aquarelle, Handzeichnungen, Lithographien. Dresden: Staatliche Kunstsammlungen.Otto Mueller (1949): Ausstellungskatalog. Berlin: Galerie Franz.Buchheim, Lothar Günther (1956): Die Künstlergemeinschaft Brücke. Feldafing.Bornschein, Rudolf &amp; Muller, Joseph-Emile (1956): Peintures, Dessins, Gravures du Musée de Sarrebruck. Nouvelles Acquisitions. Luxemburg: Musée de l'État de Luxembourg.Schmalenbach, Werner (1956): Otto Mueller. Ausstellungskatalog. Hannover: Kestner-Gesellschaft.Otto Mueller (1956): Ausstellungskatalog. Bremen: Kunsthalle Bremen.Otto Mueller (1956): Ausstellungskatalog. Hagen: Karl-Ernst-Osthaus-Museum.Otto Mueller (1957): Ausstellungskatalog. Duisburg: Städtisches Kunstmuseum Duisburg / Museumsverein Duisburg.Gemälde und Grafik aus dem Besitz des Saarlandmuseums (1957): Ausstellungskatalog. Stuttgart: Württembergischer Kunstverein.Dieck, W. (1957): Die deutschen Impressionisten und Expressionisten des Saarlandmuseums. Trier: Städtisches Museum Simeonstift.Moderne Galerie des Museums Saarbrücken (1957): Ausstellungskatalog. Opladen / Leverkusen: Städtisches Museum Leverkusen, Schloss Morsbroich.Fischer, Wend (1958): Weltausstellung Brüssel 1958 – Deutschland. Ausstellungskatalog. Brüssel: Universal and International Exhibition.Read, Herbert Edward &amp; Zeller, Alfred P. (1959): Geschichte der Modernen Malerei. München.Gombert, Hermann (1959): Von Courbet bis Miró. Freiburg: Augustinermuseum.A. B. (1959): „Saarland-Museum. Gedanken zu einer Ausstellung“. In: Saarländischer Heimat- und Kulturbund Saarheimat, 3, Saarbrücken, März 1959, S. 23.Bornschein, Rudolf (1960): „Von Renoir bis Jawlensky – Die jüngste deutsche Galerie“. In: Europa – Politik Wirtschaft Kultur, 11(3), März 1960.Buchheim, Lothar Günther (1963): Otto Mueller. Leben und Werk. Feldafing.Saarland-Museum (1963): Meisterwerke in der Kunsthalle Bremen. Bremen.Maggio Musicale Fiorentino (1964): Ausstellungskatalog. Florenz.Stadtler, Wolfgang (1964): Was sagt uns die moderne Malerei. Freiburg / Basel / Wien.Kindler Malerei Lexikon (1964): IV. Zürich.Von Courbet bis Santomaso (1966): Ausstellungskatalog. Saarbrücken: Saarlandmuseum &amp; Gebr. Röchling Bank.Moderne Galerie Saarbrücken (1968): Bestandskatalog. Saarbrücken: Saarlandmuseum, Hrsg. Rudolf Bornschein.Buchheim, Lothar Günther (1968): Otto Mueller. Reprint von 1963. Feldafing, S. 57.Landesanstalt für Erziehung und Unterricht (1968): Meisterwerke der Kunst, 16, Stuttgart, Nr. 9.Bornschein, Rudolf (1971): „Das Saarland-Museum in Saarbrücken“. In: Die Kunst und das schöne Heim, 83(6), München, S. 341.Der Neue Brockhaus (1974): Band 3. Wiesbaden.Maler und Werk (1974): Dresden.Bornschein, Rudolf (1976): Moderne Galerie Saarbrücken. Saarbrücken: Saarlandmuseum.Dittmann, Lorenz / Költzsch, Erika S. / Költzsch, Georg W. (1980): Künstler der Brücke. Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff. Gemälde, Aquarelle, Zeichnungen, Druckgraphik 1909–1930. Saarbrücken: Saarlandmuseum, Hrsg. Georg W. Költzsch, S. 172.Moderne Galerie im Saarland-Museum Saarbrücken (1981): Museumsführer. Braunschweig: Saarlandmuseum.Jähner, Horst (1986): Künstlergruppe „Brücke“. Geschichte einer Gemeinschaft. Berlin, S. 454.Elger, Dietmar (1988): Expressionismus. Eine deutsche Kunstrevolution. Köln, S. 100.Decker, Marlene (1993): Gestaltungselemente im Bildwerk von Otto Mueller. Dortmund, S. 97.Lüttichau, Mario-Andreas von (1993): Otto Mueller. Ein Romantiker unter den Expressionisten. Köln, S. 128.Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie (1995): Grenzenlos. Terminales / L / ES &amp; S / Allemand. Paris.Jähner, Horst (1996): Künstlergruppe „Brücke“, Geschichte einer Gemeinschaft und das Lebenswerk ihrer Repräsentanten. Berlin: Henschel-Verlag, S. 240.Meisterwerke des 20. Jahrhunderts – Saarland Museum Saarbrücken (1999): Bestandskatalog. Ostfildern: Saarlandmuseum, Hrsg. Ernst-Gerhard Güse, S. 86.Saarland Museum Saarbrücken (1999): In: Prestel-Museumsführer, Hrsg. Ernst-Gerhard Güse. München / London / New York, S. 37.Lüttichau, Mario-Andreas von &amp; Pirsig, Tanja (2003): Otto Mueller. Werkverzeichnis. München.Die Brücke in der Südsee – Exotik der Farbe (2005): Ausstellungskatalog. Saarbrücken: Saarland Museum, Hrsg. Ralph Melcher, S. 220.Ich sehe was, was Du nicht siehst (2014): Ausstellungskatalog. Dillingen: Gesellschaft zur Förderung des Saarländischen Kulturbesitzes e. V., Hrsg. Inge Weber, S. 211.Elvers-Svamberk, Kathrin, Janzing, Godehard, Mönig, Roland, Stocker, Mona, Uthemann, Ernest W., Müller, Alexandra (2016): Entre deux horizons. Avant-gardes allemands et françaises du Saarlandmuseum. Metz: Saarlandmuseum / Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.Augustin, Roland, Elvers-Svamberk, Kathrin, Mönig, Roland, Stocker, Mona, Uthemann, Ernest, Wolf, Eva (2017): Saarlandmuseum – Moderne Galerie: Die Sammlung. Saarbrücken: Saarlandmuseum, Hrsg. Roland Mönig, S. 94.Quarantäne (2020): S. 108.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ausstellungen / Aufführungen / Veröffentlichungen</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Ausstellung: Neue Kunst in der Orangerie, 1929.06.01.-1929.09.01., KasselAusstellung: German Painting and Sculpture, 1931.03.13.-1931.04.26., New YorkAusstellung: Allgemeine Deutsche Kunstausstellung, 1946.08.25.-1946.10.31., DresdenAusstellung: Otto Mueller, 1874-1930, 1947.09, DresdenAusstellung: Otto Mueller, 1874-1930, 1947, ChemnitzAusstellung: Otto Mueller zum 75. Geburtstag, 1949, BerlinAusstellung: Neuerwerbungen des Saarland-Museums, 1955.07.06.-1955.10.09., SaarbrückenAusstellung: Peintures, Dessins, Gravures du Musée de Sarrebruck, 1956.03.17.-1956.04.08., LuxembourgAusstellung: Otto Mueller, 1956.09.18.-1956.10.21., HannoverAusstellung: Otto Mueller, 1956, BremenAusstellung: Otto Mueller, 1956.12.09.-1957.01.13., HagenAusstellung: Otto Mueller, 1957.01.26.-1957.02.24., DuisburgAusstellung: Moderne Galerie des Museums Saarbrücken, 1957.06.04.-1957.07.07., LeverkusenAusstellung: Das Pferd in der bildenden Kunst, 1957.08.03.-1957.09.12., Baden-BadenAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, MannheimAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, FreiburgAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957.09.13.-1957.10.13., TrierAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957.07.20.-1957.09.01., StuttgartAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, KarlsruheAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, LudwigshafenAusstellung: Weltausstellung, 1958.04.18.-1958.10.19., BrüsselAusstellung: Von Courbet bis Miró, 1959.04.12.-1959.08.30., FreiburgAusstellung: Deutsche Expressionisten aus Eigenbesitz, 1961.05.08.-1961.09.20., SaarbrückenAusstellung: Saarland-Museum, 1963.04.07.-1963.06.03., BremenAusstellung: Mostra dell´ espressionismo, 1964.05.-1964.06., FlorenzAusstellung: Künstler der Brücke, 1980.10.03.-1980.11.23., SaarbrückenAusstellung: Die Brücke in der Südsee, 2005.10.22.-2006.01.08., SaarbrückenAusstellung: Entre deux horizons / Zwischen zwei Horizonten, 2016.06.29.-2017.01.16., Metz</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Objekt- oder Werkteil</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Vollständiges Werk</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Rechte / Lizenzen</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Digitalisat-Link/Pfad</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://prometheus.uni-koeln.de/rack-images/saarbruecken_ifk/original/MDAwLzAwNi85ODUvaW1hZ2UuanBn?_asd=1753719040cb8cb5b85e81e374bd46dc829ad9f681f990d74e</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Metadaten-Status</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Erfasst von</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Stefan Binder</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Erfassungsdatum</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2025-07-28 00:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Kommentar / Anmerkung</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Versionsgeschichte</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
red light works but export does not
</commit_message>
<xml_diff>
--- a/objekt_data.xlsx
+++ b/objekt_data.xlsx
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Zigeunerinnen mit Sonnenblumen</t>
+          <t>test</t>
         </is>
       </c>
     </row>
@@ -446,7 +446,11 @@
           <t>Künstler*in/Autor*in</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -454,7 +458,11 @@
           <t>Sichtbare oder genannte Personen</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -462,11 +470,7 @@
           <t>Entstehungsjahr</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1927</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -474,11 +478,7 @@
           <t>Ort der Entstehung / Nutzung</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Unbekannt</t>
-        </is>
-      </c>
+      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -494,11 +494,7 @@
           <t>Technik</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Leimfarbe, Rupfen</t>
-        </is>
-      </c>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -530,11 +526,7 @@
           <t>Narrative / Diskurse</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Darstellung von alternativen Leben fernab der Mehrheitsgesellschaft. Romantisierung des Landlebens. </t>
-        </is>
-      </c>
+      <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -542,11 +534,7 @@
           <t>Historischer Kontext</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Otto Mueller war Mitglied der expressionistischen Künstlergruppe Brücke, die sich bewusst gegen akademische Kunstkonventionen stellte. Er suchte nach Ursprünglichkeit, Einfachheit und "Naturverbundenheit" – Werte, die viele Expressionisten romantisch mit nicht-bürgerlichen oder „exotischen“ Gruppen wie z.B. den Roma verbanden.In den 1920er Jahren, in der Weimarer Republik, waren Romnja gesellschaftlich stark marginalisiert. Sie wurden überwacht, ausgegrenzt und kriminalisiert. Die Tendenzen des aufkommenden Nationalsozialismus sind zur Entstehungszeit des Bilds schon deutlich. Mueller hatte persönliche Kontakte zu einer Roma-Gruppe in Schlesien, mit der er wiederholt reiste.</t>
-        </is>
-      </c>
+      <c r="B13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -562,11 +550,7 @@
           <t>Agency</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Die Figuren sind nicht karikiert oder grotesk. Darstellung von Fürsorge und Wärme. Kind ist Zentrum einer familiären Handlung. </t>
-        </is>
-      </c>
+      <c r="B15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -606,11 +590,7 @@
           <t>Provenienz</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Vorbesitzer: Köln, Galerie Aenne AbelsVorbesitzer: Berlin, Mueller, Maschka</t>
-        </is>
-      </c>
+      <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -618,11 +598,7 @@
           <t>Literatur</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Neue Kunst in der Orangerie (1929): Vierte große Kunstausstellung Kassel. Ausstellungskatalog. Kassel: Kunstverein Kassel.Barr, Alfred H. (1931): German Painting and Sculpture. Ausstellungskatalog. New York: Museum of Modern Art.Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F. u. a. (Hrsg.) (1931): Museum der Gegenwart. Zeitschrift der deutschen Museen für neuere Kunst, 1., 2. Berlin.Allgemeine deutsche Kunstausstellung (1946). [o. Verlagsort].Balzer, Wolfgang (1947): Otto Mueller, 1874–1930. Gemälde, Aquarelle, Handzeichnungen, Lithographien. Dresden: Staatliche Kunstsammlungen.Otto Mueller (1949): Ausstellungskatalog. Berlin: Galerie Franz.Buchheim, Lothar Günther (1956): Die Künstlergemeinschaft Brücke. Feldafing.Bornschein, Rudolf &amp; Muller, Joseph-Emile (1956): Peintures, Dessins, Gravures du Musée de Sarrebruck. Nouvelles Acquisitions. Luxemburg: Musée de l'État de Luxembourg.Schmalenbach, Werner (1956): Otto Mueller. Ausstellungskatalog. Hannover: Kestner-Gesellschaft.Otto Mueller (1956): Ausstellungskatalog. Bremen: Kunsthalle Bremen.Otto Mueller (1956): Ausstellungskatalog. Hagen: Karl-Ernst-Osthaus-Museum.Otto Mueller (1957): Ausstellungskatalog. Duisburg: Städtisches Kunstmuseum Duisburg / Museumsverein Duisburg.Gemälde und Grafik aus dem Besitz des Saarlandmuseums (1957): Ausstellungskatalog. Stuttgart: Württembergischer Kunstverein.Dieck, W. (1957): Die deutschen Impressionisten und Expressionisten des Saarlandmuseums. Trier: Städtisches Museum Simeonstift.Moderne Galerie des Museums Saarbrücken (1957): Ausstellungskatalog. Opladen / Leverkusen: Städtisches Museum Leverkusen, Schloss Morsbroich.Fischer, Wend (1958): Weltausstellung Brüssel 1958 – Deutschland. Ausstellungskatalog. Brüssel: Universal and International Exhibition.Read, Herbert Edward &amp; Zeller, Alfred P. (1959): Geschichte der Modernen Malerei. München.Gombert, Hermann (1959): Von Courbet bis Miró. Freiburg: Augustinermuseum.A. B. (1959): „Saarland-Museum. Gedanken zu einer Ausstellung“. In: Saarländischer Heimat- und Kulturbund Saarheimat, 3, Saarbrücken, März 1959, S. 23.Bornschein, Rudolf (1960): „Von Renoir bis Jawlensky – Die jüngste deutsche Galerie“. In: Europa – Politik Wirtschaft Kultur, 11(3), März 1960.Buchheim, Lothar Günther (1963): Otto Mueller. Leben und Werk. Feldafing.Saarland-Museum (1963): Meisterwerke in der Kunsthalle Bremen. Bremen.Maggio Musicale Fiorentino (1964): Ausstellungskatalog. Florenz.Stadtler, Wolfgang (1964): Was sagt uns die moderne Malerei. Freiburg / Basel / Wien.Kindler Malerei Lexikon (1964): IV. Zürich.Von Courbet bis Santomaso (1966): Ausstellungskatalog. Saarbrücken: Saarlandmuseum &amp; Gebr. Röchling Bank.Moderne Galerie Saarbrücken (1968): Bestandskatalog. Saarbrücken: Saarlandmuseum, Hrsg. Rudolf Bornschein.Buchheim, Lothar Günther (1968): Otto Mueller. Reprint von 1963. Feldafing, S. 57.Landesanstalt für Erziehung und Unterricht (1968): Meisterwerke der Kunst, 16, Stuttgart, Nr. 9.Bornschein, Rudolf (1971): „Das Saarland-Museum in Saarbrücken“. In: Die Kunst und das schöne Heim, 83(6), München, S. 341.Der Neue Brockhaus (1974): Band 3. Wiesbaden.Maler und Werk (1974): Dresden.Bornschein, Rudolf (1976): Moderne Galerie Saarbrücken. Saarbrücken: Saarlandmuseum.Dittmann, Lorenz / Költzsch, Erika S. / Költzsch, Georg W. (1980): Künstler der Brücke. Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff. Gemälde, Aquarelle, Zeichnungen, Druckgraphik 1909–1930. Saarbrücken: Saarlandmuseum, Hrsg. Georg W. Költzsch, S. 172.Moderne Galerie im Saarland-Museum Saarbrücken (1981): Museumsführer. Braunschweig: Saarlandmuseum.Jähner, Horst (1986): Künstlergruppe „Brücke“. Geschichte einer Gemeinschaft. Berlin, S. 454.Elger, Dietmar (1988): Expressionismus. Eine deutsche Kunstrevolution. Köln, S. 100.Decker, Marlene (1993): Gestaltungselemente im Bildwerk von Otto Mueller. Dortmund, S. 97.Lüttichau, Mario-Andreas von (1993): Otto Mueller. Ein Romantiker unter den Expressionisten. Köln, S. 128.Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie (1995): Grenzenlos. Terminales / L / ES &amp; S / Allemand. Paris.Jähner, Horst (1996): Künstlergruppe „Brücke“, Geschichte einer Gemeinschaft und das Lebenswerk ihrer Repräsentanten. Berlin: Henschel-Verlag, S. 240.Meisterwerke des 20. Jahrhunderts – Saarland Museum Saarbrücken (1999): Bestandskatalog. Ostfildern: Saarlandmuseum, Hrsg. Ernst-Gerhard Güse, S. 86.Saarland Museum Saarbrücken (1999): In: Prestel-Museumsführer, Hrsg. Ernst-Gerhard Güse. München / London / New York, S. 37.Lüttichau, Mario-Andreas von &amp; Pirsig, Tanja (2003): Otto Mueller. Werkverzeichnis. München.Die Brücke in der Südsee – Exotik der Farbe (2005): Ausstellungskatalog. Saarbrücken: Saarland Museum, Hrsg. Ralph Melcher, S. 220.Ich sehe was, was Du nicht siehst (2014): Ausstellungskatalog. Dillingen: Gesellschaft zur Förderung des Saarländischen Kulturbesitzes e. V., Hrsg. Inge Weber, S. 211.Elvers-Svamberk, Kathrin, Janzing, Godehard, Mönig, Roland, Stocker, Mona, Uthemann, Ernest W., Müller, Alexandra (2016): Entre deux horizons. Avant-gardes allemands et françaises du Saarlandmuseum. Metz: Saarlandmuseum / Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.Augustin, Roland, Elvers-Svamberk, Kathrin, Mönig, Roland, Stocker, Mona, Uthemann, Ernest, Wolf, Eva (2017): Saarlandmuseum – Moderne Galerie: Die Sammlung. Saarbrücken: Saarlandmuseum, Hrsg. Roland Mönig, S. 94.Quarantäne (2020): S. 108.</t>
-        </is>
-      </c>
+      <c r="B21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -630,11 +606,7 @@
           <t>Ausstellungen / Aufführungen / Veröffentlichungen</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Ausstellung: Neue Kunst in der Orangerie, 1929.06.01.-1929.09.01., KasselAusstellung: German Painting and Sculpture, 1931.03.13.-1931.04.26., New YorkAusstellung: Allgemeine Deutsche Kunstausstellung, 1946.08.25.-1946.10.31., DresdenAusstellung: Otto Mueller, 1874-1930, 1947.09, DresdenAusstellung: Otto Mueller, 1874-1930, 1947, ChemnitzAusstellung: Otto Mueller zum 75. Geburtstag, 1949, BerlinAusstellung: Neuerwerbungen des Saarland-Museums, 1955.07.06.-1955.10.09., SaarbrückenAusstellung: Peintures, Dessins, Gravures du Musée de Sarrebruck, 1956.03.17.-1956.04.08., LuxembourgAusstellung: Otto Mueller, 1956.09.18.-1956.10.21., HannoverAusstellung: Otto Mueller, 1956, BremenAusstellung: Otto Mueller, 1956.12.09.-1957.01.13., HagenAusstellung: Otto Mueller, 1957.01.26.-1957.02.24., DuisburgAusstellung: Moderne Galerie des Museums Saarbrücken, 1957.06.04.-1957.07.07., LeverkusenAusstellung: Das Pferd in der bildenden Kunst, 1957.08.03.-1957.09.12., Baden-BadenAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, MannheimAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, FreiburgAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957.09.13.-1957.10.13., TrierAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957.07.20.-1957.09.01., StuttgartAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, KarlsruheAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, LudwigshafenAusstellung: Weltausstellung, 1958.04.18.-1958.10.19., BrüsselAusstellung: Von Courbet bis Miró, 1959.04.12.-1959.08.30., FreiburgAusstellung: Deutsche Expressionisten aus Eigenbesitz, 1961.05.08.-1961.09.20., SaarbrückenAusstellung: Saarland-Museum, 1963.04.07.-1963.06.03., BremenAusstellung: Mostra dell´ espressionismo, 1964.05.-1964.06., FlorenzAusstellung: Künstler der Brücke, 1980.10.03.-1980.11.23., SaarbrückenAusstellung: Die Brücke in der Südsee, 2005.10.22.-2006.01.08., SaarbrückenAusstellung: Entre deux horizons / Zwischen zwei Horizonten, 2016.06.29.-2017.01.16., Metz</t>
-        </is>
-      </c>
+      <c r="B22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -642,11 +614,7 @@
           <t>Objekt- oder Werkteil</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Vollständiges Werk</t>
-        </is>
-      </c>
+      <c r="B23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -662,11 +630,7 @@
           <t>Digitalisat-Link/Pfad</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>https://prometheus.uni-koeln.de/rack-images/saarbruecken_ifk/original/MDAwLzAwNi85ODUvaW1hZ2UuanBn?_asd=1753719040cb8cb5b85e81e374bd46dc829ad9f681f990d74e</t>
-        </is>
-      </c>
+      <c r="B25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -682,11 +646,7 @@
           <t>Erfasst von</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Stefan Binder</t>
-        </is>
-      </c>
+      <c r="B27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -694,11 +654,7 @@
           <t>Erfassungsdatum</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>2025-07-28 00:00:00</t>
-        </is>
-      </c>
+      <c r="B28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">

</xml_diff>

<commit_message>
working version for import and traffic lights
</commit_message>
<xml_diff>
--- a/objekt_data.xlsx
+++ b/objekt_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,11 @@
           <t>Value</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -436,7 +441,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>Zigeunerinnen mit Sonnenblumen</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>red</t>
         </is>
       </c>
     </row>
@@ -451,6 +461,11 @@
           <t>test</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -460,7 +475,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>aamam</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>red</t>
         </is>
       </c>
     </row>
@@ -470,7 +490,16 @@
           <t>Entstehungsjahr</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1927</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -478,7 +507,16 @@
           <t>Ort der Entstehung / Nutzung</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Unbekannt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -486,7 +524,16 @@
           <t>Gattung / Genre</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Gruppenporträt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -494,7 +541,16 @@
           <t>Technik</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Leimfarbe, Rupfen</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -503,6 +559,11 @@
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -511,6 +572,11 @@
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -518,7 +584,16 @@
           <t>Motive / Topoi</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Naturverbundenheit, Familienband</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -526,7 +601,16 @@
           <t>Narrative / Diskurse</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Darstellung von alternativen Leben fernab der Mehrheitsgesellschaft. Romantisierung des Landlebens.</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -534,7 +618,16 @@
           <t>Historischer Kontext</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Otto Mueller war Mitglied der expressionistischen Künstlergruppe Brücke, die sich bewusst gegen akademische Kunstkonventionen stellte. Er suchte nach Ursprünglichkeit, Einfachheit und "Naturverbundenheit" – Werte, die viele Expressionisten romantisch mit nicht-bürgerlichen oder „exotischen“ Gruppen wie z.B. den Roma verbanden.In den 1920er Jahren, in der Weimarer Republik, waren Romnja gesellschaftlich stark marginalisiert. Sie wurden überwacht, ausgegrenzt und kriminalisiert. Die Tendenzen des aufkommenden Nationalsozialismus sind zur Entstehungszeit des Bilds schon deutlich. Mueller hatte persönliche Kontakte zu einer Roma-Gruppe in Schlesien, mit der er wiederholt reiste.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -543,6 +636,11 @@
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -550,7 +648,16 @@
           <t>Agency</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Die Figuren sind nicht karikiert oder grotesk. Darstellung von Fürsorge und Wärme. Kind ist Zentrum einer familiären Handlung.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -559,6 +666,11 @@
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -567,6 +679,11 @@
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -575,6 +692,11 @@
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -583,6 +705,11 @@
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -590,7 +717,16 @@
           <t>Provenienz</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Vorbesitzer: Köln, Galerie Aenne AbelsVorbesitzer: Berlin, Mueller, Maschka</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -598,7 +734,16 @@
           <t>Literatur</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Neue Kunst in der Orangerie (1929): Vierte große Kunstausstellung Kassel. Ausstellungskatalog. Kassel: Kunstverein Kassel.Barr, Alfred H. (1931): German Painting and Sculpture. Ausstellungskatalog. New York: Museum of Modern Art.Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F. u. a. (Hrsg.) (1931): Museum der Gegenwart. Zeitschrift der deutschen Museen für neuere Kunst, 1., 2. Berlin.Allgemeine deutsche Kunstausstellung (1946). [o. Verlagsort].Balzer, Wolfgang (1947): Otto Mueller, 1874–1930. Gemälde, Aquarelle, Handzeichnungen, Lithographien. Dresden: Staatliche Kunstsammlungen.Otto Mueller (1949): Ausstellungskatalog. Berlin: Galerie Franz.Buchheim, Lothar Günther (1956): Die Künstlergemeinschaft Brücke. Feldafing.Bornschein, Rudolf &amp; Muller, Joseph-Emile (1956): Peintures, Dessins, Gravures du Musée de Sarrebruck. Nouvelles Acquisitions. Luxemburg: Musée de l'État de Luxembourg.Schmalenbach, Werner (1956): Otto Mueller. Ausstellungskatalog. Hannover: Kestner-Gesellschaft.Otto Mueller (1956): Ausstellungskatalog. Bremen: Kunsthalle Bremen.Otto Mueller (1956): Ausstellungskatalog. Hagen: Karl-Ernst-Osthaus-Museum.Otto Mueller (1957): Ausstellungskatalog. Duisburg: Städtisches Kunstmuseum Duisburg / Museumsverein Duisburg.Gemälde und Grafik aus dem Besitz des Saarlandmuseums (1957): Ausstellungskatalog. Stuttgart: Württembergischer Kunstverein.Dieck, W. (1957): Die deutschen Impressionisten und Expressionisten des Saarlandmuseums. Trier: Städtisches Museum Simeonstift.Moderne Galerie des Museums Saarbrücken (1957): Ausstellungskatalog. Opladen / Leverkusen: Städtisches Museum Leverkusen, Schloss Morsbroich.Fischer, Wend (1958): Weltausstellung Brüssel 1958 – Deutschland. Ausstellungskatalog. Brüssel: Universal and International Exhibition.Read, Herbert Edward &amp; Zeller, Alfred P. (1959): Geschichte der Modernen Malerei. München.Gombert, Hermann (1959): Von Courbet bis Miró. Freiburg: Augustinermuseum.A. B. (1959): „Saarland-Museum. Gedanken zu einer Ausstellung“. In: Saarländischer Heimat- und Kulturbund Saarheimat, 3, Saarbrücken, März 1959, S. 23.Bornschein, Rudolf (1960): „Von Renoir bis Jawlensky – Die jüngste deutsche Galerie“. In: Europa – Politik Wirtschaft Kultur, 11(3), März 1960.Buchheim, Lothar Günther (1963): Otto Mueller. Leben und Werk. Feldafing.Saarland-Museum (1963): Meisterwerke in der Kunsthalle Bremen. Bremen.Maggio Musicale Fiorentino (1964): Ausstellungskatalog. Florenz.Stadtler, Wolfgang (1964): Was sagt uns die moderne Malerei. Freiburg / Basel / Wien.Kindler Malerei Lexikon (1964): IV. Zürich.Von Courbet bis Santomaso (1966): Ausstellungskatalog. Saarbrücken: Saarlandmuseum &amp; Gebr. Röchling Bank.Moderne Galerie Saarbrücken (1968): Bestandskatalog. Saarbrücken: Saarlandmuseum, Hrsg. Rudolf Bornschein.Buchheim, Lothar Günther (1968): Otto Mueller. Reprint von 1963. Feldafing, S. 57.Landesanstalt für Erziehung und Unterricht (1968): Meisterwerke der Kunst, 16, Stuttgart, Nr. 9.Bornschein, Rudolf (1971): „Das Saarland-Museum in Saarbrücken“. In: Die Kunst und das schöne Heim, 83(6), München, S. 341.Der Neue Brockhaus (1974): Band 3. Wiesbaden.Maler und Werk (1974): Dresden.Bornschein, Rudolf (1976): Moderne Galerie Saarbrücken. Saarbrücken: Saarlandmuseum.Dittmann, Lorenz / Költzsch, Erika S. / Költzsch, Georg W. (1980): Künstler der Brücke. Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff. Gemälde, Aquarelle, Zeichnungen, Druckgraphik 1909–1930. Saarbrücken: Saarlandmuseum, Hrsg. Georg W. Költzsch, S. 172.Moderne Galerie im Saarland-Museum Saarbrücken (1981): Museumsführer. Braunschweig: Saarlandmuseum.Jähner, Horst (1986): Künstlergruppe „Brücke“. Geschichte einer Gemeinschaft. Berlin, S. 454.Elger, Dietmar (1988): Expressionismus. Eine deutsche Kunstrevolution. Köln, S. 100.Decker, Marlene (1993): Gestaltungselemente im Bildwerk von Otto Mueller. Dortmund, S. 97.Lüttichau, Mario-Andreas von (1993): Otto Mueller. Ein Romantiker unter den Expressionisten. Köln, S. 128.Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie (1995): Grenzenlos. Terminales / L / ES &amp; S / Allemand. Paris.Jähner, Horst (1996): Künstlergruppe „Brücke“, Geschichte einer Gemeinschaft und das Lebenswerk ihrer Repräsentanten. Berlin: Henschel-Verlag, S. 240.Meisterwerke des 20. Jahrhunderts – Saarland Museum Saarbrücken (1999): Bestandskatalog. Ostfildern: Saarlandmuseum, Hrsg. Ernst-Gerhard Güse, S. 86.Saarland Museum Saarbrücken (1999): In: Prestel-Museumsführer, Hrsg. Ernst-Gerhard Güse. München / London / New York, S. 37.Lüttichau, Mario-Andreas von &amp; Pirsig, Tanja (2003): Otto Mueller. Werkverzeichnis. München.Die Brücke in der Südsee – Exotik der Farbe (2005): Ausstellungskatalog. Saarbrücken: Saarland Museum, Hrsg. Ralph Melcher, S. 220.Ich sehe was, was Du nicht siehst (2014): Ausstellungskatalog. Dillingen: Gesellschaft zur Förderung des Saarländischen Kulturbesitzes e. V., Hrsg. Inge Weber, S. 211.Elvers-Svamberk, Kathrin, Janzing, Godehard, Mönig, Roland, Stocker, Mona, Uthemann, Ernest W., Müller, Alexandra (2016): Entre deux horizons. Avant-gardes allemands et françaises du Saarlandmuseum. Metz: Saarlandmuseum / Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.Augustin, Roland, Elvers-Svamberk, Kathrin, Mönig, Roland, Stocker, Mona, Uthemann, Ernest, Wolf, Eva (2017): Saarlandmuseum – Moderne Galerie: Die Sammlung. Saarbrücken: Saarlandmuseum, Hrsg. Roland Mönig, S. 94.Quarantäne (2020): S. 108.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -606,7 +751,16 @@
           <t>Ausstellungen / Aufführungen / Veröffentlichungen</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Ausstellung: Neue Kunst in der Orangerie, 1929.06.01.-1929.09.01., KasselAusstellung: German Painting and Sculpture, 1931.03.13.-1931.04.26., New YorkAusstellung: Allgemeine Deutsche Kunstausstellung, 1946.08.25.-1946.10.31., DresdenAusstellung: Otto Mueller, 1874-1930, 1947.09, DresdenAusstellung: Otto Mueller, 1874-1930, 1947, ChemnitzAusstellung: Otto Mueller zum 75. Geburtstag, 1949, BerlinAusstellung: Neuerwerbungen des Saarland-Museums, 1955.07.06.-1955.10.09., SaarbrückenAusstellung: Peintures, Dessins, Gravures du Musée de Sarrebruck, 1956.03.17.-1956.04.08., LuxembourgAusstellung: Otto Mueller, 1956.09.18.-1956.10.21., HannoverAusstellung: Otto Mueller, 1956, BremenAusstellung: Otto Mueller, 1956.12.09.-1957.01.13., HagenAusstellung: Otto Mueller, 1957.01.26.-1957.02.24., DuisburgAusstellung: Moderne Galerie des Museums Saarbrücken, 1957.06.04.-1957.07.07., LeverkusenAusstellung: Das Pferd in der bildenden Kunst, 1957.08.03.-1957.09.12., Baden-BadenAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, MannheimAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, FreiburgAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957.09.13.-1957.10.13., TrierAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957.07.20.-1957.09.01., StuttgartAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, KarlsruheAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, LudwigshafenAusstellung: Weltausstellung, 1958.04.18.-1958.10.19., BrüsselAusstellung: Von Courbet bis Miró, 1959.04.12.-1959.08.30., FreiburgAusstellung: Deutsche Expressionisten aus Eigenbesitz, 1961.05.08.-1961.09.20., SaarbrückenAusstellung: Saarland-Museum, 1963.04.07.-1963.06.03., BremenAusstellung: Mostra dell´ espressionismo, 1964.05.-1964.06., FlorenzAusstellung: Künstler der Brücke, 1980.10.03.-1980.11.23., SaarbrückenAusstellung: Die Brücke in der Südsee, 2005.10.22.-2006.01.08., SaarbrückenAusstellung: Entre deux horizons / Zwischen zwei Horizonten, 2016.06.29.-2017.01.16., Metz</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -614,7 +768,16 @@
           <t>Objekt- oder Werkteil</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Vollständiges Werk</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -623,6 +786,11 @@
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -630,7 +798,16 @@
           <t>Digitalisat-Link/Pfad</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://prometheus.uni-koeln.de/rack-images/saarbruecken_ifk/original/MDAwLzAwNi85ODUvaW1hZ2UuanBn?_asd=1753719040cb8cb5b85e81e374bd46dc829ad9f681f990d74e</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -639,6 +816,11 @@
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -646,7 +828,16 @@
           <t>Erfasst von</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Stefan Binder</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -654,7 +845,16 @@
           <t>Erfassungsdatum</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2025-07-28 00:00:00</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -663,6 +863,11 @@
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -671,6 +876,11 @@
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
name entity works app_all_ne.py
</commit_message>
<xml_diff>
--- a/objekt_data.xlsx
+++ b/objekt_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:D30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,11 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Name Entity</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -446,9 +451,10 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -456,16 +462,13 @@
           <t>Künstler*in/Autor*in</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -473,16 +476,13 @@
           <t>Sichtbare oder genannte Personen</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>aamam</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>red</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -497,9 +497,10 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -514,9 +515,10 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -531,7 +533,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Gruppenporträt</t>
         </is>
       </c>
     </row>
@@ -548,7 +555,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Leimfarbe, Rupfen</t>
         </is>
       </c>
     </row>
@@ -564,6 +576,7 @@
           <t>red</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -574,9 +587,10 @@
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -586,12 +600,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Naturverbundenheit, Familienband</t>
+          <t>Naturverbundenheit, Familienband, Berlin</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Familienband, Berlin</t>
         </is>
       </c>
     </row>
@@ -608,7 +627,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Landlebens</t>
         </is>
       </c>
     </row>
@@ -620,12 +644,19 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Otto Mueller war Mitglied der expressionistischen Künstlergruppe Brücke, die sich bewusst gegen akademische Kunstkonventionen stellte. Er suchte nach Ursprünglichkeit, Einfachheit und "Naturverbundenheit" – Werte, die viele Expressionisten romantisch mit nicht-bürgerlichen oder „exotischen“ Gruppen wie z.B. den Roma verbanden.In den 1920er Jahren, in der Weimarer Republik, waren Romnja gesellschaftlich stark marginalisiert. Sie wurden überwacht, ausgegrenzt und kriminalisiert. Die Tendenzen des aufkommenden Nationalsozialismus sind zur Entstehungszeit des Bilds schon deutlich. Mueller hatte persönliche Kontakte zu einer Roma-Gruppe in Schlesien, mit der er wiederholt reiste.</t>
+          <t>Otto Mueller war Mitglied der expressionistischen Künstlergruppe Brücke, die sich bewusst gegen akademische Kunstkonventionen stellte. Er suchte nach Ursprünglichkeit, Einfachheit und "Naturverbundenheit" – Werte, die viele Expressionisten romantisch mit nicht-bürgerlichen oder „exotischen“ Gruppen wie z.B. den Roma verbanden.
+In den 1920er Jahren, in der Weimarer Republik, waren Romnja gesellschaftlich stark marginalisiert. Sie wurden überwacht, ausgegrenzt und kriminalisiert. Die Tendenzen des aufkommenden Nationalsozialismus sind zur Entstehungszeit des Bilds schon deutlich. 
+Mueller hatte persönliche Kontakte zu einer Roma-Gruppe in Schlesien, mit der er wiederholt reiste.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Otto Mueller, Künstlergruppe Brücke, Weimarer Republik, Romnja, Bilds, Mueller, Schlesien</t>
         </is>
       </c>
     </row>
@@ -638,9 +669,10 @@
       <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -650,12 +682,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Die Figuren sind nicht karikiert oder grotesk. Darstellung von Fürsorge und Wärme. Kind ist Zentrum einer familiären Handlung.</t>
+          <t>Die [Figuren sind nicht] karikiert oder grotesk. Darstellung von Fürsorge und Wärme. Kind ist Zentrum einer familiären Handlung.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Fürsorge, Zentrum</t>
         </is>
       </c>
     </row>
@@ -671,6 +708,7 @@
           <t>red</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -684,6 +722,7 @@
           <t>red</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -697,6 +736,7 @@
           <t>red</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -710,6 +750,7 @@
           <t>red</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -719,12 +760,18 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Vorbesitzer: Köln, Galerie Aenne AbelsVorbesitzer: Berlin, Mueller, Maschka</t>
+          <t>Vorbesitzer: Köln, Galerie Aenne Abels
+Vorbesitzer: Berlin, Mueller, Maschka</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Köln, Galerie Aenne Abels, Berlin, Mueller, Maschka</t>
         </is>
       </c>
     </row>
@@ -736,12 +783,75 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Neue Kunst in der Orangerie (1929): Vierte große Kunstausstellung Kassel. Ausstellungskatalog. Kassel: Kunstverein Kassel.Barr, Alfred H. (1931): German Painting and Sculpture. Ausstellungskatalog. New York: Museum of Modern Art.Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F. u. a. (Hrsg.) (1931): Museum der Gegenwart. Zeitschrift der deutschen Museen für neuere Kunst, 1., 2. Berlin.Allgemeine deutsche Kunstausstellung (1946). [o. Verlagsort].Balzer, Wolfgang (1947): Otto Mueller, 1874–1930. Gemälde, Aquarelle, Handzeichnungen, Lithographien. Dresden: Staatliche Kunstsammlungen.Otto Mueller (1949): Ausstellungskatalog. Berlin: Galerie Franz.Buchheim, Lothar Günther (1956): Die Künstlergemeinschaft Brücke. Feldafing.Bornschein, Rudolf &amp; Muller, Joseph-Emile (1956): Peintures, Dessins, Gravures du Musée de Sarrebruck. Nouvelles Acquisitions. Luxemburg: Musée de l'État de Luxembourg.Schmalenbach, Werner (1956): Otto Mueller. Ausstellungskatalog. Hannover: Kestner-Gesellschaft.Otto Mueller (1956): Ausstellungskatalog. Bremen: Kunsthalle Bremen.Otto Mueller (1956): Ausstellungskatalog. Hagen: Karl-Ernst-Osthaus-Museum.Otto Mueller (1957): Ausstellungskatalog. Duisburg: Städtisches Kunstmuseum Duisburg / Museumsverein Duisburg.Gemälde und Grafik aus dem Besitz des Saarlandmuseums (1957): Ausstellungskatalog. Stuttgart: Württembergischer Kunstverein.Dieck, W. (1957): Die deutschen Impressionisten und Expressionisten des Saarlandmuseums. Trier: Städtisches Museum Simeonstift.Moderne Galerie des Museums Saarbrücken (1957): Ausstellungskatalog. Opladen / Leverkusen: Städtisches Museum Leverkusen, Schloss Morsbroich.Fischer, Wend (1958): Weltausstellung Brüssel 1958 – Deutschland. Ausstellungskatalog. Brüssel: Universal and International Exhibition.Read, Herbert Edward &amp; Zeller, Alfred P. (1959): Geschichte der Modernen Malerei. München.Gombert, Hermann (1959): Von Courbet bis Miró. Freiburg: Augustinermuseum.A. B. (1959): „Saarland-Museum. Gedanken zu einer Ausstellung“. In: Saarländischer Heimat- und Kulturbund Saarheimat, 3, Saarbrücken, März 1959, S. 23.Bornschein, Rudolf (1960): „Von Renoir bis Jawlensky – Die jüngste deutsche Galerie“. In: Europa – Politik Wirtschaft Kultur, 11(3), März 1960.Buchheim, Lothar Günther (1963): Otto Mueller. Leben und Werk. Feldafing.Saarland-Museum (1963): Meisterwerke in der Kunsthalle Bremen. Bremen.Maggio Musicale Fiorentino (1964): Ausstellungskatalog. Florenz.Stadtler, Wolfgang (1964): Was sagt uns die moderne Malerei. Freiburg / Basel / Wien.Kindler Malerei Lexikon (1964): IV. Zürich.Von Courbet bis Santomaso (1966): Ausstellungskatalog. Saarbrücken: Saarlandmuseum &amp; Gebr. Röchling Bank.Moderne Galerie Saarbrücken (1968): Bestandskatalog. Saarbrücken: Saarlandmuseum, Hrsg. Rudolf Bornschein.Buchheim, Lothar Günther (1968): Otto Mueller. Reprint von 1963. Feldafing, S. 57.Landesanstalt für Erziehung und Unterricht (1968): Meisterwerke der Kunst, 16, Stuttgart, Nr. 9.Bornschein, Rudolf (1971): „Das Saarland-Museum in Saarbrücken“. In: Die Kunst und das schöne Heim, 83(6), München, S. 341.Der Neue Brockhaus (1974): Band 3. Wiesbaden.Maler und Werk (1974): Dresden.Bornschein, Rudolf (1976): Moderne Galerie Saarbrücken. Saarbrücken: Saarlandmuseum.Dittmann, Lorenz / Költzsch, Erika S. / Költzsch, Georg W. (1980): Künstler der Brücke. Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff. Gemälde, Aquarelle, Zeichnungen, Druckgraphik 1909–1930. Saarbrücken: Saarlandmuseum, Hrsg. Georg W. Költzsch, S. 172.Moderne Galerie im Saarland-Museum Saarbrücken (1981): Museumsführer. Braunschweig: Saarlandmuseum.Jähner, Horst (1986): Künstlergruppe „Brücke“. Geschichte einer Gemeinschaft. Berlin, S. 454.Elger, Dietmar (1988): Expressionismus. Eine deutsche Kunstrevolution. Köln, S. 100.Decker, Marlene (1993): Gestaltungselemente im Bildwerk von Otto Mueller. Dortmund, S. 97.Lüttichau, Mario-Andreas von (1993): Otto Mueller. Ein Romantiker unter den Expressionisten. Köln, S. 128.Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie (1995): Grenzenlos. Terminales / L / ES &amp; S / Allemand. Paris.Jähner, Horst (1996): Künstlergruppe „Brücke“, Geschichte einer Gemeinschaft und das Lebenswerk ihrer Repräsentanten. Berlin: Henschel-Verlag, S. 240.Meisterwerke des 20. Jahrhunderts – Saarland Museum Saarbrücken (1999): Bestandskatalog. Ostfildern: Saarlandmuseum, Hrsg. Ernst-Gerhard Güse, S. 86.Saarland Museum Saarbrücken (1999): In: Prestel-Museumsführer, Hrsg. Ernst-Gerhard Güse. München / London / New York, S. 37.Lüttichau, Mario-Andreas von &amp; Pirsig, Tanja (2003): Otto Mueller. Werkverzeichnis. München.Die Brücke in der Südsee – Exotik der Farbe (2005): Ausstellungskatalog. Saarbrücken: Saarland Museum, Hrsg. Ralph Melcher, S. 220.Ich sehe was, was Du nicht siehst (2014): Ausstellungskatalog. Dillingen: Gesellschaft zur Förderung des Saarländischen Kulturbesitzes e. V., Hrsg. Inge Weber, S. 211.Elvers-Svamberk, Kathrin, Janzing, Godehard, Mönig, Roland, Stocker, Mona, Uthemann, Ernest W., Müller, Alexandra (2016): Entre deux horizons. Avant-gardes allemands et françaises du Saarlandmuseum. Metz: Saarlandmuseum / Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.Augustin, Roland, Elvers-Svamberk, Kathrin, Mönig, Roland, Stocker, Mona, Uthemann, Ernest, Wolf, Eva (2017): Saarlandmuseum – Moderne Galerie: Die Sammlung. Saarbrücken: Saarlandmuseum, Hrsg. Roland Mönig, S. 94.Quarantäne (2020): S. 108.</t>
+          <t>Neue Kunst in der Orangerie (1929): Vierte große Kunstausstellung Kassel. Ausstellungskatalog. Kassel: Kunstverein Kassel.
+Barr, Alfred H. (1931): German Painting and Sculpture. Ausstellungskatalog. New York: Museum of Modern Art.
+Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F. u. a. (Hrsg.) (1931): Museum der Gegenwart. Zeitschrift der deutschen Museen für neuere Kunst, 1., 2. Berlin.
+Allgemeine deutsche Kunstausstellung (1946). [o. Verlagsort].
+Balzer, Wolfgang (1947): Otto Mueller, 1874–1930. Gemälde, Aquarelle, Handzeichnungen, Lithographien. Dresden: Staatliche Kunstsammlungen.
+Otto Mueller (1949): Ausstellungskatalog. Berlin: Galerie Franz.
+Buchheim, Lothar Günther (1956): Die Künstlergemeinschaft Brücke. Feldafing.
+Bornschein, Rudolf &amp; Muller, Joseph-Emile (1956): Peintures, Dessins, Gravures du Musée de Sarrebruck. Nouvelles Acquisitions. Luxemburg: Musée de l'État de Luxembourg.
+Schmalenbach, Werner (1956): Otto Mueller. Ausstellungskatalog. Hannover: Kestner-Gesellschaft.
+Otto Mueller (1956): Ausstellungskatalog. Bremen: Kunsthalle Bremen.
+Otto Mueller (1956): Ausstellungskatalog. Hagen: Karl-Ernst-Osthaus-Museum.
+Otto Mueller (1957): Ausstellungskatalog. Duisburg: Städtisches Kunstmuseum Duisburg / Museumsverein Duisburg.
+Gemälde und Grafik aus dem Besitz des Saarlandmuseums (1957): Ausstellungskatalog. Stuttgart: Württembergischer Kunstverein.
+Dieck, W. (1957): Die deutschen Impressionisten und Expressionisten des Saarlandmuseums. Trier: Städtisches Museum Simeonstift.
+Moderne Galerie des Museums Saarbrücken (1957): Ausstellungskatalog. Opladen / Leverkusen: Städtisches Museum Leverkusen, Schloss Morsbroich.
+Fischer, Wend (1958): Weltausstellung Brüssel 1958 – Deutschland. Ausstellungskatalog. Brüssel: Universal and International Exhibition.
+Read, Herbert Edward &amp; Zeller, Alfred P. (1959): Geschichte der Modernen Malerei. München.
+Gombert, Hermann (1959): Von Courbet bis Miró. Freiburg: Augustinermuseum.
+A. B. (1959): „Saarland-Museum. Gedanken zu einer Ausstellung“. In: Saarländischer Heimat- und Kulturbund Saarheimat, 3, Saarbrücken, März 1959, S. 23.
+Bornschein, Rudolf (1960): „Von Renoir bis Jawlensky – Die jüngste deutsche Galerie“. In: Europa – Politik Wirtschaft Kultur, 11(3), März 1960.
+Buchheim, Lothar Günther (1963): Otto Mueller. Leben und Werk. Feldafing.
+Saarland-Museum (1963): Meisterwerke in der Kunsthalle Bremen. Bremen.
+Maggio Musicale Fiorentino (1964): Ausstellungskatalog. Florenz.
+Stadtler, Wolfgang (1964): Was sagt uns die moderne Malerei. Freiburg / Basel / Wien.
+Kindler Malerei Lexikon (1964): IV. Zürich.
+Von Courbet bis Santomaso (1966): Ausstellungskatalog. Saarbrücken: Saarlandmuseum &amp; Gebr. Röchling Bank.
+Moderne Galerie Saarbrücken (1968): Bestandskatalog. Saarbrücken: Saarlandmuseum, Hrsg. Rudolf Bornschein.
+Buchheim, Lothar Günther (1968): Otto Mueller. Reprint von 1963. Feldafing, S. 57.
+Landesanstalt für Erziehung und Unterricht (1968): Meisterwerke der Kunst, 16, Stuttgart, Nr. 9.
+Bornschein, Rudolf (1971): „Das Saarland-Museum in Saarbrücken“. In: Die Kunst und das schöne Heim, 83(6), München, S. 341.
+Der Neue Brockhaus (1974): Band 3. Wiesbaden.
+Maler und Werk (1974): Dresden.
+Bornschein, Rudolf (1976): Moderne Galerie Saarbrücken. Saarbrücken: Saarlandmuseum.
+Dittmann, Lorenz / Költzsch, Erika S. / Költzsch, Georg W. (1980): Künstler der Brücke. Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff. Gemälde, Aquarelle, Zeichnungen, Druckgraphik 1909–1930. Saarbrücken: Saarlandmuseum, Hrsg. Georg W. Költzsch, S. 172.
+Moderne Galerie im Saarland-Museum Saarbrücken (1981): Museumsführer. Braunschweig: Saarlandmuseum.
+Jähner, Horst (1986): Künstlergruppe „Brücke“. Geschichte einer Gemeinschaft. Berlin, S. 454.
+Elger, Dietmar (1988): Expressionismus. Eine deutsche Kunstrevolution. Köln, S. 100.
+Decker, Marlene (1993): Gestaltungselemente im Bildwerk von Otto Mueller. Dortmund, S. 97.
+Lüttichau, Mario-Andreas von (1993): Otto Mueller. Ein Romantiker unter den Expressionisten. Köln, S. 128.
+Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie (1995): Grenzenlos. Terminales / L / ES &amp; S / Allemand. Paris.
+Jähner, Horst (1996): Künstlergruppe „Brücke“, Geschichte einer Gemeinschaft und das Lebenswerk ihrer Repräsentanten. Berlin: Henschel-Verlag, S. 240.
+Meisterwerke des 20. Jahrhunderts – Saarland Museum Saarbrücken (1999): Bestandskatalog. Ostfildern: Saarlandmuseum, Hrsg. Ernst-Gerhard Güse, S. 86.
+Saarland Museum Saarbrücken (1999): In: Prestel-Museumsführer, Hrsg. Ernst-Gerhard Güse. München / London / New York, S. 37.
+Lüttichau, Mario-Andreas von &amp; Pirsig, Tanja (2003): Otto Mueller. Werkverzeichnis. München.
+Die Brücke in der Südsee – Exotik der Farbe (2005): Ausstellungskatalog. Saarbrücken: Saarland Museum, Hrsg. Ralph Melcher, S. 220.
+Ich sehe was, was Du nicht siehst (2014): Ausstellungskatalog. Dillingen: Gesellschaft zur Förderung des Saarländischen Kulturbesitzes e. V., Hrsg. Inge Weber, S. 211.
+Elvers-Svamberk, Kathrin, Janzing, Godehard, Mönig, Roland, Stocker, Mona, Uthemann, Ernest W., Müller, Alexandra (2016): Entre deux horizons. Avant-gardes allemands et françaises du Saarlandmuseum. Metz: Saarlandmuseum / Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.
+Augustin, Roland, Elvers-Svamberk, Kathrin, Mönig, Roland, Stocker, Mona, Uthemann, Ernest, Wolf, Eva (2017): Saarlandmuseum – Moderne Galerie: Die Sammlung. Saarbrücken: Saarlandmuseum, Hrsg. Roland Mönig, S. 94.
+Quarantäne (2020): S. 108.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Orangerie, Kassel, Kassel, Kunstverein Kassel, Barr, Alfred H., ): German Painting and Sculpture, New York, Museum of Modern Art, Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F., Hrsg., ): Museum, Balzer, Wolfgang, Otto Mueller, Handzeichnungen, Lithographien, Dresden, Otto Mueller, Berlin, Galerie Franz, Lothar Günther, Künstlergemeinschaft Brücke, Feldafing, Rudolf &amp; Muller, Joseph-Emile, ): Peintures, Dessins, Gravures du Musée de Sarrebruck, Nouvelles Acquisitions, Luxemburg, Musée de l'État de Luxembourg, Schmalenbach, Werner, Otto Mueller, Hannover, Kestner-Gesellschaft, Otto Mueller, Bremen, Kunsthalle Bremen, Otto Mueller, Hagen, Karl-Ernst-Osthaus-Museum, Otto Mueller, Duisburg, Museumsverein Duisburg, Stuttgart, Württembergischer Kunstverein, W., Trier, Städtisches Museum Simeonstift, Opladen, Leverkusen, Städtisches Museum Leverkusen, Schloss Morsbroich, Wend, Brüssel, Deutschland, Brüssel, Universal and International Exhibition, Read, Herbert Edward, Alfred P., München, Gombert, Hermann, Courbet, Miró, Freiburg: Augustinermuseum, A. B., Saarländischer Heimat- und Kulturbund, Saarbrücken, Rudolf, Renoir, Jawlensky, Europa, Lothar Günther, Otto Mueller, Feldafing, Kunsthalle Bremen, Bremen, Maggio Musicale Fiorentino, Florenz, Stadtler, Wolfgang, Freiburg, Basel, Wien, Malerei Lexikon, ): IV. Zürich, Courbet, Santomaso, Saarlandmuseum &amp; Gebr. Röchling Bank, Galerie Saarbrücken, ): Bestandskatalog, Saarbrücken, Saarlandmuseum, Hrsg., Rudolf Bornschein, Buchheim, Lothar Günther, Otto Mueller, Reprint von 1963., S., Landesanstalt für Erziehung und Unterricht, Stuttgart, Nr. 9.
+Bornschein, Rudolf, Saarland-Museum, Saarbrücken, München, S. 341.
+Der Neue Brockhaus, Rudolf, Galerie Saarbrücken, Saarbrücken, Saarlandmuseum, Dittmann, Lorenz, Költzsch, Erika S. /, Költzsch, Georg W., Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff, Saarbrücken, Saarlandmuseum, Hrsg., Georg W. Költzsch, Saarland-Museum Saarbrücken, Braunschweig, Saarlandmuseum, Jähner, Berlin, S. 454.
+, Dietmar, Köln, S. 100.
+Decker, Marlene, Otto Mueller, Dortmund, S. 97.
+Lüttichau, Mario-Andreas, Otto Mueller, Köln, S. 128.
+Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie, ): Grenzenlos, Terminales, ES &amp; S, Allemand, Paris, Jähner, Berlin, Henschel-Verlag, Saarlandmuseum, Hrsg., Ernst-Gerhard Güse, S. 86., Prestel-Museumsführer, Ernst-Gerhard Güse, München, London, New York, S. 37.
+Lüttichau, Mario-Andreas, Otto Mueller, Werkverzeichnis, München, Saarbrücken, Saarland Museum, Hrsg., Ralph Melcher, Du, ): Ausstellungskatalog, Gesellschaft zur Förderung des, Hrsg., Inge Weber, S. 211.
+Elvers-Svamberk, Godehard, Mönig, Mona, Uthemann, Ernest W., Alexandra, ): Entre deux horizons, allemands et françaises du Saarlandmuseum, Metz, Saarlandmuseum, Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.
+, Roland, Elvers-Svamberk, Mona, Uthemann, Ernest, Wolf, Saarbrücken, Saarlandmuseum, Hrsg., Roland Mönig, S. 94.
+Quarantäne, ): S. 108.</t>
         </is>
       </c>
     </row>
@@ -753,12 +863,44 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ausstellung: Neue Kunst in der Orangerie, 1929.06.01.-1929.09.01., KasselAusstellung: German Painting and Sculpture, 1931.03.13.-1931.04.26., New YorkAusstellung: Allgemeine Deutsche Kunstausstellung, 1946.08.25.-1946.10.31., DresdenAusstellung: Otto Mueller, 1874-1930, 1947.09, DresdenAusstellung: Otto Mueller, 1874-1930, 1947, ChemnitzAusstellung: Otto Mueller zum 75. Geburtstag, 1949, BerlinAusstellung: Neuerwerbungen des Saarland-Museums, 1955.07.06.-1955.10.09., SaarbrückenAusstellung: Peintures, Dessins, Gravures du Musée de Sarrebruck, 1956.03.17.-1956.04.08., LuxembourgAusstellung: Otto Mueller, 1956.09.18.-1956.10.21., HannoverAusstellung: Otto Mueller, 1956, BremenAusstellung: Otto Mueller, 1956.12.09.-1957.01.13., HagenAusstellung: Otto Mueller, 1957.01.26.-1957.02.24., DuisburgAusstellung: Moderne Galerie des Museums Saarbrücken, 1957.06.04.-1957.07.07., LeverkusenAusstellung: Das Pferd in der bildenden Kunst, 1957.08.03.-1957.09.12., Baden-BadenAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, MannheimAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, FreiburgAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957.09.13.-1957.10.13., TrierAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957.07.20.-1957.09.01., StuttgartAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, KarlsruheAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, LudwigshafenAusstellung: Weltausstellung, 1958.04.18.-1958.10.19., BrüsselAusstellung: Von Courbet bis Miró, 1959.04.12.-1959.08.30., FreiburgAusstellung: Deutsche Expressionisten aus Eigenbesitz, 1961.05.08.-1961.09.20., SaarbrückenAusstellung: Saarland-Museum, 1963.04.07.-1963.06.03., BremenAusstellung: Mostra dell´ espressionismo, 1964.05.-1964.06., FlorenzAusstellung: Künstler der Brücke, 1980.10.03.-1980.11.23., SaarbrückenAusstellung: Die Brücke in der Südsee, 2005.10.22.-2006.01.08., SaarbrückenAusstellung: Entre deux horizons / Zwischen zwei Horizonten, 2016.06.29.-2017.01.16., Metz</t>
+          <t>Ausstellung: Neue Kunst in der Orangerie, 1929.06.01.-1929.09.01., Kassel
+Ausstellung: German Painting and Sculpture, 1931.03.13.-1931.04.26., New York
+Ausstellung: Allgemeine Deutsche Kunstausstellung, 1946.08.25.-1946.10.31., Dresden
+Ausstellung: Otto Mueller, 1874-1930, 1947.09, Dresden
+Ausstellung: Otto Mueller, 1874-1930, 1947, Chemnitz
+Ausstellung: Otto Mueller zum 75. Geburtstag, 1949, Berlin
+Ausstellung: Neuerwerbungen des Saarland-Museums, 1955.07.06.-1955.10.09., Saarbrücken
+Ausstellung: Peintures, Dessins, Gravures du Musée de Sarrebruck, 1956.03.17.-1956.04.08., Luxembourg
+Ausstellung: Otto Mueller, 1956.09.18.-1956.10.21., Hannover
+Ausstellung: Otto Mueller, 1956, Bremen
+Ausstellung: Otto Mueller, 1956.12.09.-1957.01.13., Hagen
+Ausstellung: Otto Mueller, 1957.01.26.-1957.02.24., Duisburg
+Ausstellung: Moderne Galerie des Museums Saarbrücken, 1957.06.04.-1957.07.07., Leverkusen
+Ausstellung: Das Pferd in der bildenden Kunst, 1957.08.03.-1957.09.12., Baden-Baden
+Ausstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, Mannheim
+Ausstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, Freiburg
+Ausstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957.09.13.-1957.10.13., Trier
+Ausstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957.07.20.-1957.09.01., Stuttgart
+Ausstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, Karlsruhe
+Ausstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, Ludwigshafen
+Ausstellung: Weltausstellung, 1958.04.18.-1958.10.19., Brüssel
+Ausstellung: Von Courbet bis Miró, 1959.04.12.-1959.08.30., Freiburg
+Ausstellung: Deutsche Expressionisten aus Eigenbesitz, 1961.05.08.-1961.09.20., Saarbrücken
+Ausstellung: Saarland-Museum, 1963.04.07.-1963.06.03., Bremen
+Ausstellung: Mostra dell´ espressionismo, 1964.05.-1964.06., Florenz
+Ausstellung: Künstler der Brücke, 1980.10.03.-1980.11.23., Saarbrücken
+Ausstellung: Die Brücke in der Südsee, 2005.10.22.-2006.01.08., Saarbrücken
+Ausstellung: Entre deux horizons / Zwischen zwei Horizonten, 2016.06.29.-2017.01.16., Metz</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Orangerie, Kassel, German Painting and Sculpture, New York, Dresden, Otto Mueller, Dresden, Otto Mueller, Chemnitz, Otto Mueller, Berlin, Saarbrücken, Peintures, Dessins, Gravures du Musée de Sarrebruck, Luxembourg, Otto Mueller, Hannover, Otto Mueller, Bremen, Otto Mueller, Hagen, Otto Mueller, Duisburg, Museums Saarbrücken, 1957.06.04.-1957.07.07., Leverkusen, Baden-Baden, Mannheim, Freiburg, Trier, Stuttgart, Ludwigshafen, Brüssel, Courbet, Miró, 1959.04.12.-1959.08.30., Freiburg, Eigenbesitz, Saarbrücken, Bremen, Florenz, Saarbrücken, Südsee, 2005.10.22.-2006.01.08., Saarbrücken, Metz</t>
         </is>
       </c>
     </row>
@@ -775,7 +917,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Vollständiges</t>
         </is>
       </c>
     </row>
@@ -788,9 +935,10 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -805,7 +953,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://prometheus.uni-koeln.de/rack-images/saarbruecken_ifk/original/MDAwLzAwNi85ODUvaW1hZ2UuanBn?_asd=1753719040cb8cb5b85e81e374bd46dc829ad9f681f990d74e</t>
         </is>
       </c>
     </row>
@@ -821,6 +974,7 @@
           <t>red</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -835,7 +989,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Stefan Binder</t>
         </is>
       </c>
     </row>
@@ -852,9 +1011,10 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -865,9 +1025,10 @@
       <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -881,6 +1042,7 @@
           <t>red</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
name entity button works now.  app_all_button.py
</commit_message>
<xml_diff>
--- a/objekt_data.xlsx
+++ b/objekt_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,7 +533,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -545,49 +545,53 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Technik</t>
+          <t>focus_field</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Leimfarbe, Rupfen</t>
+          <t>Gattung / Genre</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Leimfarbe, Rupfen</t>
-        </is>
-      </c>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dimensionen</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
+          <t>Technik</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Leimfarbe, Rupfen</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Leimfarbe, Rupfen</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Kurzbeschreibung</t>
+          <t>Dimensionen</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>yellow</t>
+          <t>red</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -595,125 +599,123 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Motive / Topoi</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Naturverbundenheit, Familienband, Berlin</t>
-        </is>
-      </c>
+          <t>Kurzbeschreibung</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Familienband, Berlin</t>
-        </is>
-      </c>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Narrative / Diskurse</t>
+          <t>Motive / Topoi</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Darstellung von alternativen Leben fernab der Mehrheitsgesellschaft. Romantisierung des Landlebens.</t>
+          <t>Naturverbundenheit, Familienband, Berlin</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Landlebens</t>
+          <t>Familienband, Berlin</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Historischer Kontext</t>
+          <t>Narrative / Diskurse</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Otto Mueller war Mitglied der expressionistischen Künstlergruppe Brücke, die sich bewusst gegen akademische Kunstkonventionen stellte. Er suchte nach Ursprünglichkeit, Einfachheit und "Naturverbundenheit" – Werte, die viele Expressionisten romantisch mit nicht-bürgerlichen oder „exotischen“ Gruppen wie z.B. den Roma verbanden.
-In den 1920er Jahren, in der Weimarer Republik, waren Romnja gesellschaftlich stark marginalisiert. Sie wurden überwacht, ausgegrenzt und kriminalisiert. Die Tendenzen des aufkommenden Nationalsozialismus sind zur Entstehungszeit des Bilds schon deutlich. 
-Mueller hatte persönliche Kontakte zu einer Roma-Gruppe in Schlesien, mit der er wiederholt reiste.</t>
+          <t>Darstellung von alternativen Leben fernab der Mehrheitsgesellschaft. Romantisierung des Landlebens.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Otto Mueller, Künstlergruppe Brücke, Weimarer Republik, Romnja, Bilds, Mueller, Schlesien</t>
+          <t>Landlebens</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Antiziganistische / Stigmatisierende Elemente</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
+          <t>Historischer Kontext</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Otto Mueller war Mitglied der expressionistischen Künstlergruppe Brücke, die sich bewusst gegen akademische Kunstkonventionen stellte. Er suchte nach Ursprünglichkeit, Einfachheit und "Naturverbundenheit" – Werte, die viele Expressionisten romantisch mit nicht-bürgerlichen oder „exotischen“ Gruppen wie z.B. den Roma verbanden.In den 1920er Jahren, in der Weimarer Republik, waren Romnja gesellschaftlich stark marginalisiert. Sie wurden überwacht, ausgegrenzt und kriminalisiert. Die Tendenzen des aufkommenden Nationalsozialismus sind zur Entstehungszeit des Bilds schon deutlich. Mueller hatte persönliche Kontakte zu einer Roma-Gruppe in Schlesien, mit der er wiederholt reiste.</t>
+        </is>
+      </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>yellow</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Otto Mueller, Künstlergruppe Brücke, Weimarer Republik, Romnja, Bilds, Mueller, Schlesien</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Agency</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Die [Figuren sind nicht] karikiert oder grotesk. Darstellung von Fürsorge und Wärme. Kind ist Zentrum einer familiären Handlung.</t>
-        </is>
-      </c>
+          <t>Antiziganistische / Stigmatisierende Elemente</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Fürsorge, Zentrum</t>
-        </is>
-      </c>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Verknüpfung</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
+          <t>Agency</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Die [Figuren sind nicht] karikiert oder grotesk. Darstellung von Fürsorge und Wärme. Kind ist Zentrum einer familiären Handlung.</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Fürsorge, Zentrum</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Narrativwandel bei Medienwechsel</t>
+          <t>Verknüpfung</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -727,7 +729,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Rezeptionsweg</t>
+          <t>Narrativwandel bei Medienwechsel</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -741,13 +743,13 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sammlung / Archiv</t>
+          <t>Rezeptionsweg</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
@@ -755,258 +757,164 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Provenienz</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Vorbesitzer: Köln, Galerie Aenne Abels
-Vorbesitzer: Berlin, Mueller, Maschka</t>
-        </is>
-      </c>
+          <t>Sammlung / Archiv</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Köln, Galerie Aenne Abels, Berlin, Mueller, Maschka</t>
-        </is>
-      </c>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Literatur</t>
+          <t>Provenienz</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Neue Kunst in der Orangerie (1929): Vierte große Kunstausstellung Kassel. Ausstellungskatalog. Kassel: Kunstverein Kassel.
-Barr, Alfred H. (1931): German Painting and Sculpture. Ausstellungskatalog. New York: Museum of Modern Art.
-Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F. u. a. (Hrsg.) (1931): Museum der Gegenwart. Zeitschrift der deutschen Museen für neuere Kunst, 1., 2. Berlin.
-Allgemeine deutsche Kunstausstellung (1946). [o. Verlagsort].
-Balzer, Wolfgang (1947): Otto Mueller, 1874–1930. Gemälde, Aquarelle, Handzeichnungen, Lithographien. Dresden: Staatliche Kunstsammlungen.
-Otto Mueller (1949): Ausstellungskatalog. Berlin: Galerie Franz.
-Buchheim, Lothar Günther (1956): Die Künstlergemeinschaft Brücke. Feldafing.
-Bornschein, Rudolf &amp; Muller, Joseph-Emile (1956): Peintures, Dessins, Gravures du Musée de Sarrebruck. Nouvelles Acquisitions. Luxemburg: Musée de l'État de Luxembourg.
-Schmalenbach, Werner (1956): Otto Mueller. Ausstellungskatalog. Hannover: Kestner-Gesellschaft.
-Otto Mueller (1956): Ausstellungskatalog. Bremen: Kunsthalle Bremen.
-Otto Mueller (1956): Ausstellungskatalog. Hagen: Karl-Ernst-Osthaus-Museum.
-Otto Mueller (1957): Ausstellungskatalog. Duisburg: Städtisches Kunstmuseum Duisburg / Museumsverein Duisburg.
-Gemälde und Grafik aus dem Besitz des Saarlandmuseums (1957): Ausstellungskatalog. Stuttgart: Württembergischer Kunstverein.
-Dieck, W. (1957): Die deutschen Impressionisten und Expressionisten des Saarlandmuseums. Trier: Städtisches Museum Simeonstift.
-Moderne Galerie des Museums Saarbrücken (1957): Ausstellungskatalog. Opladen / Leverkusen: Städtisches Museum Leverkusen, Schloss Morsbroich.
-Fischer, Wend (1958): Weltausstellung Brüssel 1958 – Deutschland. Ausstellungskatalog. Brüssel: Universal and International Exhibition.
-Read, Herbert Edward &amp; Zeller, Alfred P. (1959): Geschichte der Modernen Malerei. München.
-Gombert, Hermann (1959): Von Courbet bis Miró. Freiburg: Augustinermuseum.
-A. B. (1959): „Saarland-Museum. Gedanken zu einer Ausstellung“. In: Saarländischer Heimat- und Kulturbund Saarheimat, 3, Saarbrücken, März 1959, S. 23.
-Bornschein, Rudolf (1960): „Von Renoir bis Jawlensky – Die jüngste deutsche Galerie“. In: Europa – Politik Wirtschaft Kultur, 11(3), März 1960.
-Buchheim, Lothar Günther (1963): Otto Mueller. Leben und Werk. Feldafing.
-Saarland-Museum (1963): Meisterwerke in der Kunsthalle Bremen. Bremen.
-Maggio Musicale Fiorentino (1964): Ausstellungskatalog. Florenz.
-Stadtler, Wolfgang (1964): Was sagt uns die moderne Malerei. Freiburg / Basel / Wien.
-Kindler Malerei Lexikon (1964): IV. Zürich.
-Von Courbet bis Santomaso (1966): Ausstellungskatalog. Saarbrücken: Saarlandmuseum &amp; Gebr. Röchling Bank.
-Moderne Galerie Saarbrücken (1968): Bestandskatalog. Saarbrücken: Saarlandmuseum, Hrsg. Rudolf Bornschein.
-Buchheim, Lothar Günther (1968): Otto Mueller. Reprint von 1963. Feldafing, S. 57.
-Landesanstalt für Erziehung und Unterricht (1968): Meisterwerke der Kunst, 16, Stuttgart, Nr. 9.
-Bornschein, Rudolf (1971): „Das Saarland-Museum in Saarbrücken“. In: Die Kunst und das schöne Heim, 83(6), München, S. 341.
-Der Neue Brockhaus (1974): Band 3. Wiesbaden.
-Maler und Werk (1974): Dresden.
-Bornschein, Rudolf (1976): Moderne Galerie Saarbrücken. Saarbrücken: Saarlandmuseum.
-Dittmann, Lorenz / Költzsch, Erika S. / Költzsch, Georg W. (1980): Künstler der Brücke. Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff. Gemälde, Aquarelle, Zeichnungen, Druckgraphik 1909–1930. Saarbrücken: Saarlandmuseum, Hrsg. Georg W. Költzsch, S. 172.
-Moderne Galerie im Saarland-Museum Saarbrücken (1981): Museumsführer. Braunschweig: Saarlandmuseum.
-Jähner, Horst (1986): Künstlergruppe „Brücke“. Geschichte einer Gemeinschaft. Berlin, S. 454.
-Elger, Dietmar (1988): Expressionismus. Eine deutsche Kunstrevolution. Köln, S. 100.
-Decker, Marlene (1993): Gestaltungselemente im Bildwerk von Otto Mueller. Dortmund, S. 97.
-Lüttichau, Mario-Andreas von (1993): Otto Mueller. Ein Romantiker unter den Expressionisten. Köln, S. 128.
-Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie (1995): Grenzenlos. Terminales / L / ES &amp; S / Allemand. Paris.
-Jähner, Horst (1996): Künstlergruppe „Brücke“, Geschichte einer Gemeinschaft und das Lebenswerk ihrer Repräsentanten. Berlin: Henschel-Verlag, S. 240.
-Meisterwerke des 20. Jahrhunderts – Saarland Museum Saarbrücken (1999): Bestandskatalog. Ostfildern: Saarlandmuseum, Hrsg. Ernst-Gerhard Güse, S. 86.
-Saarland Museum Saarbrücken (1999): In: Prestel-Museumsführer, Hrsg. Ernst-Gerhard Güse. München / London / New York, S. 37.
-Lüttichau, Mario-Andreas von &amp; Pirsig, Tanja (2003): Otto Mueller. Werkverzeichnis. München.
-Die Brücke in der Südsee – Exotik der Farbe (2005): Ausstellungskatalog. Saarbrücken: Saarland Museum, Hrsg. Ralph Melcher, S. 220.
-Ich sehe was, was Du nicht siehst (2014): Ausstellungskatalog. Dillingen: Gesellschaft zur Förderung des Saarländischen Kulturbesitzes e. V., Hrsg. Inge Weber, S. 211.
-Elvers-Svamberk, Kathrin, Janzing, Godehard, Mönig, Roland, Stocker, Mona, Uthemann, Ernest W., Müller, Alexandra (2016): Entre deux horizons. Avant-gardes allemands et françaises du Saarlandmuseum. Metz: Saarlandmuseum / Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.
-Augustin, Roland, Elvers-Svamberk, Kathrin, Mönig, Roland, Stocker, Mona, Uthemann, Ernest, Wolf, Eva (2017): Saarlandmuseum – Moderne Galerie: Die Sammlung. Saarbrücken: Saarlandmuseum, Hrsg. Roland Mönig, S. 94.
-Quarantäne (2020): S. 108.</t>
+          <t>Vorbesitzer: Köln, Galerie Aenne AbelsVorbesitzer: Berlin, Mueller, Maschka</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Orangerie, Kassel, Kassel, Kunstverein Kassel, Barr, Alfred H., ): German Painting and Sculpture, New York, Museum of Modern Art, Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F., Hrsg., ): Museum, Balzer, Wolfgang, Otto Mueller, Handzeichnungen, Lithographien, Dresden, Otto Mueller, Berlin, Galerie Franz, Lothar Günther, Künstlergemeinschaft Brücke, Feldafing, Rudolf &amp; Muller, Joseph-Emile, ): Peintures, Dessins, Gravures du Musée de Sarrebruck, Nouvelles Acquisitions, Luxemburg, Musée de l'État de Luxembourg, Schmalenbach, Werner, Otto Mueller, Hannover, Kestner-Gesellschaft, Otto Mueller, Bremen, Kunsthalle Bremen, Otto Mueller, Hagen, Karl-Ernst-Osthaus-Museum, Otto Mueller, Duisburg, Museumsverein Duisburg, Stuttgart, Württembergischer Kunstverein, W., Trier, Städtisches Museum Simeonstift, Opladen, Leverkusen, Städtisches Museum Leverkusen, Schloss Morsbroich, Wend, Brüssel, Deutschland, Brüssel, Universal and International Exhibition, Read, Herbert Edward, Alfred P., München, Gombert, Hermann, Courbet, Miró, Freiburg: Augustinermuseum, A. B., Saarländischer Heimat- und Kulturbund, Saarbrücken, Rudolf, Renoir, Jawlensky, Europa, Lothar Günther, Otto Mueller, Feldafing, Kunsthalle Bremen, Bremen, Maggio Musicale Fiorentino, Florenz, Stadtler, Wolfgang, Freiburg, Basel, Wien, Malerei Lexikon, ): IV. Zürich, Courbet, Santomaso, Saarlandmuseum &amp; Gebr. Röchling Bank, Galerie Saarbrücken, ): Bestandskatalog, Saarbrücken, Saarlandmuseum, Hrsg., Rudolf Bornschein, Buchheim, Lothar Günther, Otto Mueller, Reprint von 1963., S., Landesanstalt für Erziehung und Unterricht, Stuttgart, Nr. 9.
-Bornschein, Rudolf, Saarland-Museum, Saarbrücken, München, S. 341.
-Der Neue Brockhaus, Rudolf, Galerie Saarbrücken, Saarbrücken, Saarlandmuseum, Dittmann, Lorenz, Költzsch, Erika S. /, Költzsch, Georg W., Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff, Saarbrücken, Saarlandmuseum, Hrsg., Georg W. Költzsch, Saarland-Museum Saarbrücken, Braunschweig, Saarlandmuseum, Jähner, Berlin, S. 454.
-, Dietmar, Köln, S. 100.
-Decker, Marlene, Otto Mueller, Dortmund, S. 97.
-Lüttichau, Mario-Andreas, Otto Mueller, Köln, S. 128.
-Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie, ): Grenzenlos, Terminales, ES &amp; S, Allemand, Paris, Jähner, Berlin, Henschel-Verlag, Saarlandmuseum, Hrsg., Ernst-Gerhard Güse, S. 86., Prestel-Museumsführer, Ernst-Gerhard Güse, München, London, New York, S. 37.
-Lüttichau, Mario-Andreas, Otto Mueller, Werkverzeichnis, München, Saarbrücken, Saarland Museum, Hrsg., Ralph Melcher, Du, ): Ausstellungskatalog, Gesellschaft zur Förderung des, Hrsg., Inge Weber, S. 211.
-Elvers-Svamberk, Godehard, Mönig, Mona, Uthemann, Ernest W., Alexandra, ): Entre deux horizons, allemands et françaises du Saarlandmuseum, Metz, Saarlandmuseum, Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.
-, Roland, Elvers-Svamberk, Mona, Uthemann, Ernest, Wolf, Saarbrücken, Saarlandmuseum, Hrsg., Roland Mönig, S. 94.
-Quarantäne, ): S. 108.</t>
+          <t>Köln, Galerie Aenne, AbelsVorbesitzer, Berlin, Mueller, Maschka</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ausstellungen / Aufführungen / Veröffentlichungen</t>
+          <t>Literatur</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ausstellung: Neue Kunst in der Orangerie, 1929.06.01.-1929.09.01., Kassel
-Ausstellung: German Painting and Sculpture, 1931.03.13.-1931.04.26., New York
-Ausstellung: Allgemeine Deutsche Kunstausstellung, 1946.08.25.-1946.10.31., Dresden
-Ausstellung: Otto Mueller, 1874-1930, 1947.09, Dresden
-Ausstellung: Otto Mueller, 1874-1930, 1947, Chemnitz
-Ausstellung: Otto Mueller zum 75. Geburtstag, 1949, Berlin
-Ausstellung: Neuerwerbungen des Saarland-Museums, 1955.07.06.-1955.10.09., Saarbrücken
-Ausstellung: Peintures, Dessins, Gravures du Musée de Sarrebruck, 1956.03.17.-1956.04.08., Luxembourg
-Ausstellung: Otto Mueller, 1956.09.18.-1956.10.21., Hannover
-Ausstellung: Otto Mueller, 1956, Bremen
-Ausstellung: Otto Mueller, 1956.12.09.-1957.01.13., Hagen
-Ausstellung: Otto Mueller, 1957.01.26.-1957.02.24., Duisburg
-Ausstellung: Moderne Galerie des Museums Saarbrücken, 1957.06.04.-1957.07.07., Leverkusen
-Ausstellung: Das Pferd in der bildenden Kunst, 1957.08.03.-1957.09.12., Baden-Baden
-Ausstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, Mannheim
-Ausstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, Freiburg
-Ausstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957.09.13.-1957.10.13., Trier
-Ausstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957.07.20.-1957.09.01., Stuttgart
-Ausstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, Karlsruhe
-Ausstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, Ludwigshafen
-Ausstellung: Weltausstellung, 1958.04.18.-1958.10.19., Brüssel
-Ausstellung: Von Courbet bis Miró, 1959.04.12.-1959.08.30., Freiburg
-Ausstellung: Deutsche Expressionisten aus Eigenbesitz, 1961.05.08.-1961.09.20., Saarbrücken
-Ausstellung: Saarland-Museum, 1963.04.07.-1963.06.03., Bremen
-Ausstellung: Mostra dell´ espressionismo, 1964.05.-1964.06., Florenz
-Ausstellung: Künstler der Brücke, 1980.10.03.-1980.11.23., Saarbrücken
-Ausstellung: Die Brücke in der Südsee, 2005.10.22.-2006.01.08., Saarbrücken
-Ausstellung: Entre deux horizons / Zwischen zwei Horizonten, 2016.06.29.-2017.01.16., Metz</t>
+          <t>Neue Kunst in der Orangerie (1929): Vierte große Kunstausstellung Kassel. Ausstellungskatalog. Kassel: Kunstverein Kassel.Barr, Alfred H. (1931): German Painting and Sculpture. Ausstellungskatalog. New York: Museum of Modern Art.Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F. u. a. (Hrsg.) (1931): Museum der Gegenwart. Zeitschrift der deutschen Museen für neuere Kunst, 1., 2. Berlin.Allgemeine deutsche Kunstausstellung (1946). [o. Verlagsort].Balzer, Wolfgang (1947): Otto Mueller, 1874–1930. Gemälde, Aquarelle, Handzeichnungen, Lithographien. Dresden: Staatliche Kunstsammlungen.Otto Mueller (1949): Ausstellungskatalog. Berlin: Galerie Franz.Buchheim, Lothar Günther (1956): Die Künstlergemeinschaft Brücke. Feldafing.Bornschein, Rudolf &amp; Muller, Joseph-Emile (1956): Peintures, Dessins, Gravures du Musée de Sarrebruck. Nouvelles Acquisitions. Luxemburg: Musée de l'État de Luxembourg.Schmalenbach, Werner (1956): Otto Mueller. Ausstellungskatalog. Hannover: Kestner-Gesellschaft.Otto Mueller (1956): Ausstellungskatalog. Bremen: Kunsthalle Bremen.Otto Mueller (1956): Ausstellungskatalog. Hagen: Karl-Ernst-Osthaus-Museum.Otto Mueller (1957): Ausstellungskatalog. Duisburg: Städtisches Kunstmuseum Duisburg / Museumsverein Duisburg.Gemälde und Grafik aus dem Besitz des Saarlandmuseums (1957): Ausstellungskatalog. Stuttgart: Württembergischer Kunstverein.Dieck, W. (1957): Die deutschen Impressionisten und Expressionisten des Saarlandmuseums. Trier: Städtisches Museum Simeonstift.Moderne Galerie des Museums Saarbrücken (1957): Ausstellungskatalog. Opladen / Leverkusen: Städtisches Museum Leverkusen, Schloss Morsbroich.Fischer, Wend (1958): Weltausstellung Brüssel 1958 – Deutschland. Ausstellungskatalog. Brüssel: Universal and International Exhibition.Read, Herbert Edward &amp; Zeller, Alfred P. (1959): Geschichte der Modernen Malerei. München.Gombert, Hermann (1959): Von Courbet bis Miró. Freiburg: Augustinermuseum.A. B. (1959): „Saarland-Museum. Gedanken zu einer Ausstellung“. In: Saarländischer Heimat- und Kulturbund Saarheimat, 3, Saarbrücken, März 1959, S. 23.Bornschein, Rudolf (1960): „Von Renoir bis Jawlensky – Die jüngste deutsche Galerie“. In: Europa – Politik Wirtschaft Kultur, 11(3), März 1960.Buchheim, Lothar Günther (1963): Otto Mueller. Leben und Werk. Feldafing.Saarland-Museum (1963): Meisterwerke in der Kunsthalle Bremen. Bremen.Maggio Musicale Fiorentino (1964): Ausstellungskatalog. Florenz.Stadtler, Wolfgang (1964): Was sagt uns die moderne Malerei. Freiburg / Basel / Wien.Kindler Malerei Lexikon (1964): IV. Zürich.Von Courbet bis Santomaso (1966): Ausstellungskatalog. Saarbrücken: Saarlandmuseum &amp; Gebr. Röchling Bank.Moderne Galerie Saarbrücken (1968): Bestandskatalog. Saarbrücken: Saarlandmuseum, Hrsg. Rudolf Bornschein.Buchheim, Lothar Günther (1968): Otto Mueller. Reprint von 1963. Feldafing, S. 57.Landesanstalt für Erziehung und Unterricht (1968): Meisterwerke der Kunst, 16, Stuttgart, Nr. 9.Bornschein, Rudolf (1971): „Das Saarland-Museum in Saarbrücken“. In: Die Kunst und das schöne Heim, 83(6), München, S. 341.Der Neue Brockhaus (1974): Band 3. Wiesbaden.Maler und Werk (1974): Dresden.Bornschein, Rudolf (1976): Moderne Galerie Saarbrücken. Saarbrücken: Saarlandmuseum.Dittmann, Lorenz / Költzsch, Erika S. / Költzsch, Georg W. (1980): Künstler der Brücke. Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff. Gemälde, Aquarelle, Zeichnungen, Druckgraphik 1909–1930. Saarbrücken: Saarlandmuseum, Hrsg. Georg W. Költzsch, S. 172.Moderne Galerie im Saarland-Museum Saarbrücken (1981): Museumsführer. Braunschweig: Saarlandmuseum.Jähner, Horst (1986): Künstlergruppe „Brücke“. Geschichte einer Gemeinschaft. Berlin, S. 454.Elger, Dietmar (1988): Expressionismus. Eine deutsche Kunstrevolution. Köln, S. 100.Decker, Marlene (1993): Gestaltungselemente im Bildwerk von Otto Mueller. Dortmund, S. 97.Lüttichau, Mario-Andreas von (1993): Otto Mueller. Ein Romantiker unter den Expressionisten. Köln, S. 128.Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie (1995): Grenzenlos. Terminales / L / ES &amp; S / Allemand. Paris.Jähner, Horst (1996): Künstlergruppe „Brücke“, Geschichte einer Gemeinschaft und das Lebenswerk ihrer Repräsentanten. Berlin: Henschel-Verlag, S. 240.Meisterwerke des 20. Jahrhunderts – Saarland Museum Saarbrücken (1999): Bestandskatalog. Ostfildern: Saarlandmuseum, Hrsg. Ernst-Gerhard Güse, S. 86.Saarland Museum Saarbrücken (1999): In: Prestel-Museumsführer, Hrsg. Ernst-Gerhard Güse. München / London / New York, S. 37.Lüttichau, Mario-Andreas von &amp; Pirsig, Tanja (2003): Otto Mueller. Werkverzeichnis. München.Die Brücke in der Südsee – Exotik der Farbe (2005): Ausstellungskatalog. Saarbrücken: Saarland Museum, Hrsg. Ralph Melcher, S. 220.Ich sehe was, was Du nicht siehst (2014): Ausstellungskatalog. Dillingen: Gesellschaft zur Förderung des Saarländischen Kulturbesitzes e. V., Hrsg. Inge Weber, S. 211.Elvers-Svamberk, Kathrin, Janzing, Godehard, Mönig, Roland, Stocker, Mona, Uthemann, Ernest W., Müller, Alexandra (2016): Entre deux horizons. Avant-gardes allemands et françaises du Saarlandmuseum. Metz: Saarlandmuseum / Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.Augustin, Roland, Elvers-Svamberk, Kathrin, Mönig, Roland, Stocker, Mona, Uthemann, Ernest, Wolf, Eva (2017): Saarlandmuseum – Moderne Galerie: Die Sammlung. Saarbrücken: Saarlandmuseum, Hrsg. Roland Mönig, S. 94.Quarantäne (2020): S. 108.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Orangerie, Kassel, German Painting and Sculpture, New York, Dresden, Otto Mueller, Dresden, Otto Mueller, Chemnitz, Otto Mueller, Berlin, Saarbrücken, Peintures, Dessins, Gravures du Musée de Sarrebruck, Luxembourg, Otto Mueller, Hannover, Otto Mueller, Bremen, Otto Mueller, Hagen, Otto Mueller, Duisburg, Museums Saarbrücken, 1957.06.04.-1957.07.07., Leverkusen, Baden-Baden, Mannheim, Freiburg, Trier, Stuttgart, Ludwigshafen, Brüssel, Courbet, Miró, 1959.04.12.-1959.08.30., Freiburg, Eigenbesitz, Saarbrücken, Bremen, Florenz, Saarbrücken, Südsee, 2005.10.22.-2006.01.08., Saarbrücken, Metz</t>
+          <t>Orangerie, Kassel, Kassel, Kunstverein Kassel, Barr, Alfred H., ): German Painting and Sculpture, New York, Museum of Modern Art, Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F., Hrsg., ): Museum, Wolfgang, Otto Mueller, Handzeichnungen, Lithographien, Dresden, Otto Mueller, Berlin, Galerie Franz, Buchheim, Lothar Günther, Künstlergemeinschaft Brücke, Feldafing, Rudolf &amp; Muller, Joseph-Emile, ): Peintures, Dessins, Gravures du Musée de Sarrebruck, Nouvelles Acquisitions, Luxemburg, Musée de l'État de Luxembourg, Schmalenbach, Werner, Otto Mueller, Hannover, Kestner-Gesellschaft, Otto Mueller, Bremen, Kunsthalle Bremen, Otto Mueller, Hagen, Karl-Ernst-Osthaus-Museum, Otto Mueller, Duisburg, Museumsverein Duisburg, Stuttgart, Württembergischer Kunstverein, Dieck, W., Trier, Städtisches Museum Simeonstift, Museums Saarbrücken, Opladen, Leverkusen, Städtisches Museum Leverkusen, Schloss Morsbroich, Wend, Brüssel, Deutschland, Brüssel, Universal and International Exhibition, Read, Herbert Edward, Alfred P., München, Gombert, Hermann, Courbet, Miró, Freiburg: Augustinermuseum, A. B., Saarländischer Heimat- und Kulturbund, Saarbrücken, S. 23.Bornschein, Rudolf, Renoir, Jawlensky, Europa, Lothar Günther, Otto Mueller, Feldafing, Kunsthalle Bremen, Bremen, Maggio Musicale Fiorentino, Florenz, Stadtler, Wolfgang, Freiburg, Basel, Wien, ): IV. Zürich, Courbet, Santomaso, Saarlandmuseum &amp; Gebr. Röchling Bank, Galerie Saarbrücken, ): Bestandskatalog, Saarbrücken, Saarlandmuseum, Hrsg., Rudolf Bornschein, Buchheim, Lothar Günther, Otto Mueller, Reprint von 1963., S., Stuttgart, Nr. 9.Bornschein, Rudolf, Saarland-Museum, Saarbrücken, München, S. 341.Der Neue Brockhaus, ): Dresden, Bornschein, Rudolf, Galerie Saarbrücken, Saarbrücken, Saarlandmuseum, Dittmann, Lorenz, Költzsch, Erika S. /, Költzsch, Georg W., Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff, Saarbrücken, Saarlandmuseum, Hrsg., Georg W. Költzsch, S. 172.Moderne, Saarland-Museum Saarbrücken, Braunschweig, Saarlandmuseum, Jähner, Berlin, S. 454.Elger, Dietmar, Köln, S. 100.Decker, Marlene, ): Gestaltungselemente, Otto Mueller, Dortmund, S. 97.Lüttichau, Mario-Andreas, Otto Mueller, Köln, S. 128.Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie, ): Grenzenlos, Terminales, ES &amp; S, Allemand, Paris, Jähner, Berlin, Henschel-Verlag, Saarlandmuseum, Hrsg., Ernst-Gerhard Güse, Museum Saarbrücken, Prestel-Museumsführer, Ernst-Gerhard Güse, München, London, New York, S. 37.Lüttichau, Mario-Andreas, Otto Mueller, Werkverzeichnis, München, Saarbrücken, Saarland Museum, Hrsg., Ralph Melcher, S. 220.Ich, Du, ): Ausstellungskatalog, Gesellschaft zur Förderung des, Hrsg., Inge Weber, Godehard, Mönig, Mona, Uthemann, Ernest W., Alexandra, ): Entre deux horizons, allemands et françaises du Saarlandmuseum, Metz, Saarlandmuseum, Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.Augustin, Roland, Mona, Uthemann, Ernest, Wolf, Saarbrücken, Saarlandmuseum, Hrsg., Roland Mönig, S. 94.Quarantäne, ): S. 108.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Objekt- oder Werkteil</t>
+          <t>Ausstellungen / Aufführungen / Veröffentlichungen</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Vollständiges Werk</t>
+          <t>Ausstellung: Neue Kunst in der Orangerie, 1929.06.01.-1929.09.01., KasselAusstellung: German Painting and Sculpture, 1931.03.13.-1931.04.26., New YorkAusstellung: Allgemeine Deutsche Kunstausstellung, 1946.08.25.-1946.10.31., DresdenAusstellung: Otto Mueller, 1874-1930, 1947.09, DresdenAusstellung: Otto Mueller, 1874-1930, 1947, ChemnitzAusstellung: Otto Mueller zum 75. Geburtstag, 1949, BerlinAusstellung: Neuerwerbungen des Saarland-Museums, 1955.07.06.-1955.10.09., SaarbrückenAusstellung: Peintures, Dessins, Gravures du Musée de Sarrebruck, 1956.03.17.-1956.04.08., LuxembourgAusstellung: Otto Mueller, 1956.09.18.-1956.10.21., HannoverAusstellung: Otto Mueller, 1956, BremenAusstellung: Otto Mueller, 1956.12.09.-1957.01.13., HagenAusstellung: Otto Mueller, 1957.01.26.-1957.02.24., DuisburgAusstellung: Moderne Galerie des Museums Saarbrücken, 1957.06.04.-1957.07.07., LeverkusenAusstellung: Das Pferd in der bildenden Kunst, 1957.08.03.-1957.09.12., Baden-BadenAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, MannheimAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, FreiburgAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957.09.13.-1957.10.13., TrierAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957.07.20.-1957.09.01., StuttgartAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, KarlsruheAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, LudwigshafenAusstellung: Weltausstellung, 1958.04.18.-1958.10.19., BrüsselAusstellung: Von Courbet bis Miró, 1959.04.12.-1959.08.30., FreiburgAusstellung: Deutsche Expressionisten aus Eigenbesitz, 1961.05.08.-1961.09.20., SaarbrückenAusstellung: Saarland-Museum, 1963.04.07.-1963.06.03., BremenAusstellung: Mostra dell´ espressionismo, 1964.05.-1964.06., FlorenzAusstellung: Künstler der Brücke, 1980.10.03.-1980.11.23., SaarbrückenAusstellung: Die Brücke in der Südsee, 2005.10.22.-2006.01.08., SaarbrückenAusstellung: Entre deux horizons / Zwischen zwei Horizonten, 2016.06.29.-2017.01.16., Metz</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>green</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Vollständiges</t>
+          <t>German Painting and Sculpture, DresdenAusstellung, Otto Mueller, DresdenAusstellung, Otto Mueller, ChemnitzAusstellung, Otto Mueller, SaarbrückenAusstellung, Peintures, Dessins, Gravures du Musée de Sarrebruck, Otto Mueller, HannoverAusstellung, Otto Mueller, BremenAusstellung, Otto Mueller, Otto Mueller, DuisburgAusstellung, Museums Saarbrücken, FreiburgAusstellung, TrierAusstellung, LudwigshafenAusstellung, Courbet, Miró, FreiburgAusstellung, Eigenbesitz, FlorenzAusstellung, Südsee, Metz</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Rechte / Lizenzen</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
+          <t>Objekt- oder Werkteil</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Vollständiges Werk</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>yellow</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Vollständiges</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Digitalisat-Link/Pfad</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>https://prometheus.uni-koeln.de/rack-images/saarbruecken_ifk/original/MDAwLzAwNi85ODUvaW1hZ2UuanBn?_asd=1753719040cb8cb5b85e81e374bd46dc829ad9f681f990d74e</t>
-        </is>
-      </c>
+          <t>Rechte / Lizenzen</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>https://prometheus.uni-koeln.de/rack-images/saarbruecken_ifk/original/MDAwLzAwNi85ODUvaW1hZ2UuanBn?_asd=1753719040cb8cb5b85e81e374bd46dc829ad9f681f990d74e</t>
-        </is>
-      </c>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Metadaten-Status</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
+          <t>Digitalisat-Link/Pfad</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://prometheus.uni-koeln.de/rack-images/saarbruecken_ifk/original/MDAwLzAwNi85ODUvaW1hZ2UuanBn?_asd=1753719040cb8cb5b85e81e374bd46dc829ad9f681f990d74e</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://prometheus.uni-koeln.de/rack-images/saarbruecken_ifk/original/MDAwLzAwNi85ODUvaW1hZ2UuanBn?_asd=1753719040cb8cb5b85e81e374bd46dc829ad9f681f990d74e</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Erfasst von</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Stefan Binder</t>
-        </is>
-      </c>
+          <t>Metadaten-Status</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
-          <t>green</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Stefan Binder</t>
-        </is>
-      </c>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Erfassungsdatum</t>
+          <t>Erfasst von</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2025-07-28 00:00:00</t>
+          <t>Stefan Binder</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1014,15 +922,23 @@
           <t>yellow</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Stefan Binder</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Kommentar / Anmerkung</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
+          <t>Erfassungsdatum</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2025-07-28 00:00:00</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
           <t>yellow</t>
@@ -1033,7 +949,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Versionsgeschichte</t>
+          <t>Kommentar / Anmerkung</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -1043,6 +959,20 @@
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Versionsgeschichte</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>red</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
the first column name change after import works app_all_buttons.py
</commit_message>
<xml_diff>
--- a/objekt_data.xlsx
+++ b/objekt_data.xlsx
@@ -446,7 +446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Zigeunerinnen mit Sonnenblumen</t>
+          <t>"Zigeunerpaar"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -462,13 +462,21 @@
           <t>Künstler*in/Autor*in</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Karl Friedrich Ströher</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>red</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>yellow</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Karl Friedrich Ströher</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -476,10 +484,14 @@
           <t>Sichtbare oder genannte Personen</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>unbekanntes Paar</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
@@ -492,7 +504,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1927</t>
+          <t>1912.0</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -510,7 +522,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Unbekannt</t>
+          <t>vermutlich Berlin</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -518,7 +530,11 @@
           <t>yellow</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -528,7 +544,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gruppenporträt</t>
+          <t>Bildende Kunst</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -536,11 +552,7 @@
           <t>yellow</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Gruppenporträt</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -548,11 +560,7 @@
           <t>focus_field</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Gattung / Genre</t>
-        </is>
-      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>red</t>
@@ -568,7 +576,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Leimfarbe, Rupfen</t>
+          <t>Öl Gemälde</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -576,11 +584,7 @@
           <t>yellow</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Leimfarbe, Rupfen</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -602,13 +606,21 @@
           <t>Kurzbeschreibung</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Paar in leichter Draufsicht und grellem Sonnenlicht mit Schattenpartien gezeigt. Beide tragen bunte Kleidung, die Frau in farbenfroher Tracht blickt aus dem Bild heraus, während der Mann mit Hut zu ihr schaut. Das Gemälde ist einem pointillistischen Stil, indem die Pinselschläge an Mosaik erinnern.</t>
+        </is>
+      </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>yellow</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Paar, Schattenpartien</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -618,7 +630,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Naturverbundenheit, Familienband, Berlin</t>
+          <t>Exotismus, Buntheit, Hautfarbe</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -626,11 +638,7 @@
           <t>yellow</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Familienband, Berlin</t>
-        </is>
-      </c>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -640,7 +648,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Darstellung von alternativen Leben fernab der Mehrheitsgesellschaft. Romantisierung des Landlebens.</t>
+          <t>No data</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -648,11 +656,7 @@
           <t>yellow</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Landlebens</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -662,7 +666,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Otto Mueller war Mitglied der expressionistischen Künstlergruppe Brücke, die sich bewusst gegen akademische Kunstkonventionen stellte. Er suchte nach Ursprünglichkeit, Einfachheit und "Naturverbundenheit" – Werte, die viele Expressionisten romantisch mit nicht-bürgerlichen oder „exotischen“ Gruppen wie z.B. den Roma verbanden.In den 1920er Jahren, in der Weimarer Republik, waren Romnja gesellschaftlich stark marginalisiert. Sie wurden überwacht, ausgegrenzt und kriminalisiert. Die Tendenzen des aufkommenden Nationalsozialismus sind zur Entstehungszeit des Bilds schon deutlich. Mueller hatte persönliche Kontakte zu einer Roma-Gruppe in Schlesien, mit der er wiederholt reiste.</t>
+          <t>Ströher ist Meisterschüler in Berlin und macht Reisen nach Frankreich und Spanien</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -672,7 +676,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Otto Mueller, Künstlergruppe Brücke, Weimarer Republik, Romnja, Bilds, Mueller, Schlesien</t>
+          <t>Ströher, Berlin, Frankreich, Spanien</t>
         </is>
       </c>
     </row>
@@ -682,10 +686,14 @@
           <t>Antiziganistische / Stigmatisierende Elemente</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -698,7 +706,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Die [Figuren sind nicht] karikiert oder grotesk. Darstellung von Fürsorge und Wärme. Kind ist Zentrum einer familiären Handlung.</t>
+          <t>No data</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -706,11 +714,7 @@
           <t>yellow</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Fürsorge, Zentrum</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -718,10 +722,14 @@
           <t>Verknüpfung</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -732,10 +740,14 @@
           <t>Narrativwandel bei Medienwechsel</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -746,7 +758,11 @@
           <t>Rezeptionsweg</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>yellow</t>
@@ -760,7 +776,11 @@
           <t>Sammlung / Archiv</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>yellow</t>
@@ -776,7 +796,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Vorbesitzer: Köln, Galerie Aenne AbelsVorbesitzer: Berlin, Mueller, Maschka</t>
+          <t>Möglicherweise nach Skizzen aus Spanien oder dort entstanden.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -786,7 +806,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Köln, Galerie Aenne, AbelsVorbesitzer, Berlin, Mueller, Maschka</t>
+          <t>Spanien</t>
         </is>
       </c>
     </row>
@@ -798,7 +818,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Neue Kunst in der Orangerie (1929): Vierte große Kunstausstellung Kassel. Ausstellungskatalog. Kassel: Kunstverein Kassel.Barr, Alfred H. (1931): German Painting and Sculpture. Ausstellungskatalog. New York: Museum of Modern Art.Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F. u. a. (Hrsg.) (1931): Museum der Gegenwart. Zeitschrift der deutschen Museen für neuere Kunst, 1., 2. Berlin.Allgemeine deutsche Kunstausstellung (1946). [o. Verlagsort].Balzer, Wolfgang (1947): Otto Mueller, 1874–1930. Gemälde, Aquarelle, Handzeichnungen, Lithographien. Dresden: Staatliche Kunstsammlungen.Otto Mueller (1949): Ausstellungskatalog. Berlin: Galerie Franz.Buchheim, Lothar Günther (1956): Die Künstlergemeinschaft Brücke. Feldafing.Bornschein, Rudolf &amp; Muller, Joseph-Emile (1956): Peintures, Dessins, Gravures du Musée de Sarrebruck. Nouvelles Acquisitions. Luxemburg: Musée de l'État de Luxembourg.Schmalenbach, Werner (1956): Otto Mueller. Ausstellungskatalog. Hannover: Kestner-Gesellschaft.Otto Mueller (1956): Ausstellungskatalog. Bremen: Kunsthalle Bremen.Otto Mueller (1956): Ausstellungskatalog. Hagen: Karl-Ernst-Osthaus-Museum.Otto Mueller (1957): Ausstellungskatalog. Duisburg: Städtisches Kunstmuseum Duisburg / Museumsverein Duisburg.Gemälde und Grafik aus dem Besitz des Saarlandmuseums (1957): Ausstellungskatalog. Stuttgart: Württembergischer Kunstverein.Dieck, W. (1957): Die deutschen Impressionisten und Expressionisten des Saarlandmuseums. Trier: Städtisches Museum Simeonstift.Moderne Galerie des Museums Saarbrücken (1957): Ausstellungskatalog. Opladen / Leverkusen: Städtisches Museum Leverkusen, Schloss Morsbroich.Fischer, Wend (1958): Weltausstellung Brüssel 1958 – Deutschland. Ausstellungskatalog. Brüssel: Universal and International Exhibition.Read, Herbert Edward &amp; Zeller, Alfred P. (1959): Geschichte der Modernen Malerei. München.Gombert, Hermann (1959): Von Courbet bis Miró. Freiburg: Augustinermuseum.A. B. (1959): „Saarland-Museum. Gedanken zu einer Ausstellung“. In: Saarländischer Heimat- und Kulturbund Saarheimat, 3, Saarbrücken, März 1959, S. 23.Bornschein, Rudolf (1960): „Von Renoir bis Jawlensky – Die jüngste deutsche Galerie“. In: Europa – Politik Wirtschaft Kultur, 11(3), März 1960.Buchheim, Lothar Günther (1963): Otto Mueller. Leben und Werk. Feldafing.Saarland-Museum (1963): Meisterwerke in der Kunsthalle Bremen. Bremen.Maggio Musicale Fiorentino (1964): Ausstellungskatalog. Florenz.Stadtler, Wolfgang (1964): Was sagt uns die moderne Malerei. Freiburg / Basel / Wien.Kindler Malerei Lexikon (1964): IV. Zürich.Von Courbet bis Santomaso (1966): Ausstellungskatalog. Saarbrücken: Saarlandmuseum &amp; Gebr. Röchling Bank.Moderne Galerie Saarbrücken (1968): Bestandskatalog. Saarbrücken: Saarlandmuseum, Hrsg. Rudolf Bornschein.Buchheim, Lothar Günther (1968): Otto Mueller. Reprint von 1963. Feldafing, S. 57.Landesanstalt für Erziehung und Unterricht (1968): Meisterwerke der Kunst, 16, Stuttgart, Nr. 9.Bornschein, Rudolf (1971): „Das Saarland-Museum in Saarbrücken“. In: Die Kunst und das schöne Heim, 83(6), München, S. 341.Der Neue Brockhaus (1974): Band 3. Wiesbaden.Maler und Werk (1974): Dresden.Bornschein, Rudolf (1976): Moderne Galerie Saarbrücken. Saarbrücken: Saarlandmuseum.Dittmann, Lorenz / Költzsch, Erika S. / Költzsch, Georg W. (1980): Künstler der Brücke. Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff. Gemälde, Aquarelle, Zeichnungen, Druckgraphik 1909–1930. Saarbrücken: Saarlandmuseum, Hrsg. Georg W. Költzsch, S. 172.Moderne Galerie im Saarland-Museum Saarbrücken (1981): Museumsführer. Braunschweig: Saarlandmuseum.Jähner, Horst (1986): Künstlergruppe „Brücke“. Geschichte einer Gemeinschaft. Berlin, S. 454.Elger, Dietmar (1988): Expressionismus. Eine deutsche Kunstrevolution. Köln, S. 100.Decker, Marlene (1993): Gestaltungselemente im Bildwerk von Otto Mueller. Dortmund, S. 97.Lüttichau, Mario-Andreas von (1993): Otto Mueller. Ein Romantiker unter den Expressionisten. Köln, S. 128.Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie (1995): Grenzenlos. Terminales / L / ES &amp; S / Allemand. Paris.Jähner, Horst (1996): Künstlergruppe „Brücke“, Geschichte einer Gemeinschaft und das Lebenswerk ihrer Repräsentanten. Berlin: Henschel-Verlag, S. 240.Meisterwerke des 20. Jahrhunderts – Saarland Museum Saarbrücken (1999): Bestandskatalog. Ostfildern: Saarlandmuseum, Hrsg. Ernst-Gerhard Güse, S. 86.Saarland Museum Saarbrücken (1999): In: Prestel-Museumsführer, Hrsg. Ernst-Gerhard Güse. München / London / New York, S. 37.Lüttichau, Mario-Andreas von &amp; Pirsig, Tanja (2003): Otto Mueller. Werkverzeichnis. München.Die Brücke in der Südsee – Exotik der Farbe (2005): Ausstellungskatalog. Saarbrücken: Saarland Museum, Hrsg. Ralph Melcher, S. 220.Ich sehe was, was Du nicht siehst (2014): Ausstellungskatalog. Dillingen: Gesellschaft zur Förderung des Saarländischen Kulturbesitzes e. V., Hrsg. Inge Weber, S. 211.Elvers-Svamberk, Kathrin, Janzing, Godehard, Mönig, Roland, Stocker, Mona, Uthemann, Ernest W., Müller, Alexandra (2016): Entre deux horizons. Avant-gardes allemands et françaises du Saarlandmuseum. Metz: Saarlandmuseum / Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.Augustin, Roland, Elvers-Svamberk, Kathrin, Mönig, Roland, Stocker, Mona, Uthemann, Ernest, Wolf, Eva (2017): Saarlandmuseum – Moderne Galerie: Die Sammlung. Saarbrücken: Saarlandmuseum, Hrsg. Roland Mönig, S. 94.Quarantäne (2020): S. 108.</t>
+          <t>Lebenserinnerungen des Malers Friedrich Karl Ströher 1876 - 1925, hrsg. vom Freundeskreises des Werkes Karl Friedrich Ströher und dem Hunsrück-Museum Simmern, Simmern 2004, S. 52</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -808,7 +828,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Orangerie, Kassel, Kassel, Kunstverein Kassel, Barr, Alfred H., ): German Painting and Sculpture, New York, Museum of Modern Art, Dorner, Alexander, Gosebruch, Ernst, Hartlaub, Gustav F., Hrsg., ): Museum, Wolfgang, Otto Mueller, Handzeichnungen, Lithographien, Dresden, Otto Mueller, Berlin, Galerie Franz, Buchheim, Lothar Günther, Künstlergemeinschaft Brücke, Feldafing, Rudolf &amp; Muller, Joseph-Emile, ): Peintures, Dessins, Gravures du Musée de Sarrebruck, Nouvelles Acquisitions, Luxemburg, Musée de l'État de Luxembourg, Schmalenbach, Werner, Otto Mueller, Hannover, Kestner-Gesellschaft, Otto Mueller, Bremen, Kunsthalle Bremen, Otto Mueller, Hagen, Karl-Ernst-Osthaus-Museum, Otto Mueller, Duisburg, Museumsverein Duisburg, Stuttgart, Württembergischer Kunstverein, Dieck, W., Trier, Städtisches Museum Simeonstift, Museums Saarbrücken, Opladen, Leverkusen, Städtisches Museum Leverkusen, Schloss Morsbroich, Wend, Brüssel, Deutschland, Brüssel, Universal and International Exhibition, Read, Herbert Edward, Alfred P., München, Gombert, Hermann, Courbet, Miró, Freiburg: Augustinermuseum, A. B., Saarländischer Heimat- und Kulturbund, Saarbrücken, S. 23.Bornschein, Rudolf, Renoir, Jawlensky, Europa, Lothar Günther, Otto Mueller, Feldafing, Kunsthalle Bremen, Bremen, Maggio Musicale Fiorentino, Florenz, Stadtler, Wolfgang, Freiburg, Basel, Wien, ): IV. Zürich, Courbet, Santomaso, Saarlandmuseum &amp; Gebr. Röchling Bank, Galerie Saarbrücken, ): Bestandskatalog, Saarbrücken, Saarlandmuseum, Hrsg., Rudolf Bornschein, Buchheim, Lothar Günther, Otto Mueller, Reprint von 1963., S., Stuttgart, Nr. 9.Bornschein, Rudolf, Saarland-Museum, Saarbrücken, München, S. 341.Der Neue Brockhaus, ): Dresden, Bornschein, Rudolf, Galerie Saarbrücken, Saarbrücken, Saarlandmuseum, Dittmann, Lorenz, Költzsch, Erika S. /, Költzsch, Georg W., Heckel, Kirchner, Mueller, Pechstein, Schmidt-Rottluff, Saarbrücken, Saarlandmuseum, Hrsg., Georg W. Költzsch, S. 172.Moderne, Saarland-Museum Saarbrücken, Braunschweig, Saarlandmuseum, Jähner, Berlin, S. 454.Elger, Dietmar, Köln, S. 100.Decker, Marlene, ): Gestaltungselemente, Otto Mueller, Dortmund, S. 97.Lüttichau, Mario-Andreas, Otto Mueller, Köln, S. 128.Benhamou, Brigitte, Brandts, Evelyne, Grumbach, Eric &amp; Marhuenda, Marie, ): Grenzenlos, Terminales, ES &amp; S, Allemand, Paris, Jähner, Berlin, Henschel-Verlag, Saarlandmuseum, Hrsg., Ernst-Gerhard Güse, Museum Saarbrücken, Prestel-Museumsführer, Ernst-Gerhard Güse, München, London, New York, S. 37.Lüttichau, Mario-Andreas, Otto Mueller, Werkverzeichnis, München, Saarbrücken, Saarland Museum, Hrsg., Ralph Melcher, S. 220.Ich, Du, ): Ausstellungskatalog, Gesellschaft zur Förderung des, Hrsg., Inge Weber, Godehard, Mönig, Mona, Uthemann, Ernest W., Alexandra, ): Entre deux horizons, allemands et françaises du Saarlandmuseum, Metz, Saarlandmuseum, Centre Pompidou-Metz, Hrsg. Roland Mönig, S. 197.Augustin, Roland, Mona, Uthemann, Ernest, Wolf, Saarbrücken, Saarlandmuseum, Hrsg., Roland Mönig, S. 94.Quarantäne, ): S. 108.</t>
+          <t>Friedrich Karl Ströher, Karl Friedrich Ströher, Hunsrück-Museum, Simmern, S. 52</t>
         </is>
       </c>
     </row>
@@ -820,7 +840,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Ausstellung: Neue Kunst in der Orangerie, 1929.06.01.-1929.09.01., KasselAusstellung: German Painting and Sculpture, 1931.03.13.-1931.04.26., New YorkAusstellung: Allgemeine Deutsche Kunstausstellung, 1946.08.25.-1946.10.31., DresdenAusstellung: Otto Mueller, 1874-1930, 1947.09, DresdenAusstellung: Otto Mueller, 1874-1930, 1947, ChemnitzAusstellung: Otto Mueller zum 75. Geburtstag, 1949, BerlinAusstellung: Neuerwerbungen des Saarland-Museums, 1955.07.06.-1955.10.09., SaarbrückenAusstellung: Peintures, Dessins, Gravures du Musée de Sarrebruck, 1956.03.17.-1956.04.08., LuxembourgAusstellung: Otto Mueller, 1956.09.18.-1956.10.21., HannoverAusstellung: Otto Mueller, 1956, BremenAusstellung: Otto Mueller, 1956.12.09.-1957.01.13., HagenAusstellung: Otto Mueller, 1957.01.26.-1957.02.24., DuisburgAusstellung: Moderne Galerie des Museums Saarbrücken, 1957.06.04.-1957.07.07., LeverkusenAusstellung: Das Pferd in der bildenden Kunst, 1957.08.03.-1957.09.12., Baden-BadenAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, MannheimAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957, FreiburgAusstellung: Die deutschen Impressionisten und Expressionisten des Saarlandmuseums, 1957.09.13.-1957.10.13., TrierAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957.07.20.-1957.09.01., StuttgartAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, KarlsruheAusstellung: Gemälde und Graphik aus dem Besitz des Saarlandmuseums, 1957, LudwigshafenAusstellung: Weltausstellung, 1958.04.18.-1958.10.19., BrüsselAusstellung: Von Courbet bis Miró, 1959.04.12.-1959.08.30., FreiburgAusstellung: Deutsche Expressionisten aus Eigenbesitz, 1961.05.08.-1961.09.20., SaarbrückenAusstellung: Saarland-Museum, 1963.04.07.-1963.06.03., BremenAusstellung: Mostra dell´ espressionismo, 1964.05.-1964.06., FlorenzAusstellung: Künstler der Brücke, 1980.10.03.-1980.11.23., SaarbrückenAusstellung: Die Brücke in der Südsee, 2005.10.22.-2006.01.08., SaarbrückenAusstellung: Entre deux horizons / Zwischen zwei Horizonten, 2016.06.29.-2017.01.16., Metz</t>
+          <t>"Ströher in Spanien" Simmern, 2023-2024</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -830,7 +850,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>German Painting and Sculpture, DresdenAusstellung, Otto Mueller, DresdenAusstellung, Otto Mueller, ChemnitzAusstellung, Otto Mueller, SaarbrückenAusstellung, Peintures, Dessins, Gravures du Musée de Sarrebruck, Otto Mueller, HannoverAusstellung, Otto Mueller, BremenAusstellung, Otto Mueller, Otto Mueller, DuisburgAusstellung, Museums Saarbrücken, FreiburgAusstellung, TrierAusstellung, LudwigshafenAusstellung, Courbet, Miró, FreiburgAusstellung, Eigenbesitz, FlorenzAusstellung, Südsee, Metz</t>
+          <t>Simmern</t>
         </is>
       </c>
     </row>
@@ -842,7 +862,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Vollständiges Werk</t>
+          <t>No data</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -850,11 +870,7 @@
           <t>yellow</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Vollständiges</t>
-        </is>
-      </c>
+      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -862,10 +878,14 @@
           <t>Rechte / Lizenzen</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
@@ -878,7 +898,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://prometheus.uni-koeln.de/rack-images/saarbruecken_ifk/original/MDAwLzAwNi85ODUvaW1hZ2UuanBn?_asd=1753719040cb8cb5b85e81e374bd46dc829ad9f681f990d74e</t>
+          <t>No data</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -886,11 +906,7 @@
           <t>yellow</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>https://prometheus.uni-koeln.de/rack-images/saarbruecken_ifk/original/MDAwLzAwNi85ODUvaW1hZ2UuanBn?_asd=1753719040cb8cb5b85e81e374bd46dc829ad9f681f990d74e</t>
-        </is>
-      </c>
+      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -898,10 +914,14 @@
           <t>Metadaten-Status</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -914,7 +934,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Stefan Binder</t>
+          <t>No data</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -922,11 +942,7 @@
           <t>yellow</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Stefan Binder</t>
-        </is>
-      </c>
+      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -936,7 +952,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2025-07-28 00:00:00</t>
+          <t>No data</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -952,10 +968,14 @@
           <t>Kommentar / Anmerkung</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -966,10 +986,14 @@
           <t>Versionsgeschichte</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>No data</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>red</t>
+          <t>yellow</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>

</xml_diff>